<commit_message>
13F-delta v2 complete: layer distribution refreshed
13F-delta layer now firing. Resolves issuer names via EDGAR
company_tickers index (CUSIP path was unreliable). Activist
additions weighted higher than smart-money long-term.

Refreshed layer-firing distribution after 13F:
  9L: 1 (FOUR)
  8L: 4 (was 3) -- 13F added one more
  7L: 20
  6L: 47
  5L: 94

Bearish detections (-15 cap each):
  HHH: smart money exits + activist trim
  UBER, META, GOOGL: net smart-money exits
</commit_message>
<xml_diff>
--- a/MOST_ASYMMETRIC.xlsx
+++ b/MOST_ASYMMETRIC.xlsx
@@ -152,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -221,6 +221,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -799,7 +802,7 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 6.314</t>
+          <t>9 layers firing | cons 6.502</t>
         </is>
       </c>
       <c r="F16" s="12" t="n"/>
@@ -825,7 +828,7 @@
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.618</t>
+          <t>8 layers firing | cons 7.04</t>
         </is>
       </c>
       <c r="F17" s="12" t="n"/>
@@ -836,12 +839,12 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -851,7 +854,7 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.354</t>
+          <t>8 layers firing | cons 6.79</t>
         </is>
       </c>
       <c r="F18" s="12" t="n"/>
@@ -888,22 +891,22 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>NUS</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Nu Skin</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>Named asset-sale trigger + 5-metric clean per-share stack</t>
+          <t>8 layers firing | cons 5.326</t>
         </is>
       </c>
       <c r="F20" s="12" t="n"/>
@@ -914,22 +917,22 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>NUS</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>GPGI</t>
-        </is>
-      </c>
-      <c r="D21" s="15" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>Nu Skin</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.772</t>
+          <t>Named asset-sale trigger + 5-metric clean per-share stack</t>
         </is>
       </c>
       <c r="F21" s="12" t="n"/>
@@ -940,22 +943,22 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>SBET</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>DXC Technology</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.49</t>
+          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
         </is>
       </c>
       <c r="F22" s="12" t="n"/>
@@ -966,12 +969,12 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>Universal Display</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
@@ -981,7 +984,7 @@
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
+          <t>7 layers firing | cons 5.532</t>
         </is>
       </c>
       <c r="F23" s="12" t="n"/>
@@ -992,22 +995,22 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Salesforce</t>
-        </is>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+          <t>Universal Display</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
+          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
         </is>
       </c>
       <c r="F24" s="12" t="n"/>
@@ -1018,22 +1021,22 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>HDSN</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>POOL</t>
-        </is>
-      </c>
-      <c r="D25" s="15" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>Hudson Technologies</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.354</t>
+          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
         </is>
       </c>
       <c r="F25" s="12" t="n"/>
@@ -1044,22 +1047,22 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>HUBS</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+          <t>POOL</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.352</t>
+          <t>7 layers firing | cons 5.338</t>
         </is>
       </c>
       <c r="F26" s="12" t="n"/>
@@ -1070,12 +1073,12 @@
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>DXC</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>DXC Technology</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr">
@@ -1085,7 +1088,7 @@
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
+          <t>7 layers firing | cons 5.336</t>
         </is>
       </c>
       <c r="F27" s="12" t="n"/>
@@ -1096,12 +1099,12 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>PRGO</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>PRGO</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="D28" s="16" t="inlineStr">
@@ -1111,7 +1114,7 @@
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.112</t>
+          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
         </is>
       </c>
       <c r="F28" s="12" t="n"/>
@@ -1122,12 +1125,12 @@
       </c>
       <c r="B29" s="14" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>GIII</t>
         </is>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>GIII</t>
         </is>
       </c>
       <c r="D29" s="15" t="inlineStr">
@@ -1137,7 +1140,7 @@
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.956</t>
+          <t>7 layers firing | cons 5.046</t>
         </is>
       </c>
       <c r="F29" s="12" t="n"/>
@@ -1148,22 +1151,22 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>BLND</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>GIII</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>BLND</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.914</t>
+          <t>7 layers firing | cons 5.034</t>
         </is>
       </c>
       <c r="F30" s="12" t="n"/>
@@ -1174,22 +1177,22 @@
       </c>
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>KMPR</t>
         </is>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>CERT</t>
-        </is>
-      </c>
-      <c r="D31" s="16" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+          <t>Kemper</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.876</t>
+          <t>Anti-hedge/pledge + verified buyback EXECUTING (largest verified shrinkage)</t>
         </is>
       </c>
       <c r="F31" s="12" t="n"/>
@@ -1200,22 +1203,22 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>HDSN</t>
+          <t>PRGO</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Hudson Technologies</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>PRGO</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
         <is>
-          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
+          <t>7 layers firing | cons 4.824</t>
         </is>
       </c>
       <c r="F32" s="12" t="n"/>
@@ -1226,22 +1229,22 @@
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>KMPR</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Kemper</t>
-        </is>
-      </c>
-      <c r="D33" s="15" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>LULU</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
         <is>
-          <t>Anti-hedge/pledge + verified buyback EXECUTING (largest verified shrinkage)</t>
+          <t>7 layers firing | cons 4.682</t>
         </is>
       </c>
       <c r="F33" s="12" t="n"/>
@@ -1252,22 +1255,22 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>AZTA</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>Zoetis</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.406</t>
+          <t>F4 cluster + valuation + recent-incentive 60% drawdown</t>
         </is>
       </c>
       <c r="F34" s="12" t="n"/>
@@ -1278,22 +1281,22 @@
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>CERT</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Zoetis</t>
-        </is>
-      </c>
-      <c r="D35" s="15" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>CERT</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E35" s="15" t="inlineStr">
         <is>
-          <t>F4 cluster + valuation + recent-incentive 60% drawdown</t>
+          <t>7 layers firing | cons 4.524</t>
         </is>
       </c>
       <c r="F35" s="12" t="n"/>
@@ -1423,7 +1426,7 @@
       <c r="C5" s="19" t="n">
         <v>4410</v>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="D5" s="27" t="n">
         <v>72</v>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -1449,7 +1452,7 @@
       <c r="C6" s="21" t="n">
         <v>4410</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="D6" s="27" t="n">
         <v>72</v>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -1475,7 +1478,7 @@
       <c r="C7" s="19" t="n">
         <v>6164</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="27" t="n">
         <v>100</v>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -1501,7 +1504,7 @@
       <c r="C8" s="21" t="n">
         <v>6164</v>
       </c>
-      <c r="D8" s="26" t="n">
+      <c r="D8" s="27" t="n">
         <v>100</v>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -1527,7 +1530,7 @@
       <c r="C9" s="19" t="n">
         <v>1995</v>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="30" t="n">
         <v>32</v>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -1553,7 +1556,7 @@
       <c r="C10" s="21" t="n">
         <v>2132</v>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="30" t="n">
         <v>35</v>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -1579,7 +1582,7 @@
       <c r="C11" s="19" t="n">
         <v>800</v>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="30" t="n">
         <v>13</v>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -1605,7 +1608,7 @@
       <c r="C12" s="21" t="n">
         <v>346</v>
       </c>
-      <c r="D12" s="31" t="n">
+      <c r="D12" s="32" t="n">
         <v>6</v>
       </c>
       <c r="E12" s="15" t="inlineStr">
@@ -1774,7 +1777,7 @@
           <t>Universe construction</t>
         </is>
       </c>
-      <c r="C5" s="32" t="inlineStr">
+      <c r="C5" s="33" t="inlineStr">
         <is>
           <t>6,164 US-listed common tickers from cancel_10b5_1.json — authoritative NYSE/Nasdaq/AMEX/CBOE set.</t>
         </is>
@@ -1789,7 +1792,7 @@
           <t>Layer ingestion</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="34" t="inlineStr">
         <is>
           <t>Seven scoring layers ingested per ticker: PSU forensics, governance, valuation, buyback verification, tender mechanics, 10b5-1 directional, Form 4 P-buys (plus Form 144 for bearish).</t>
         </is>
@@ -1804,7 +1807,7 @@
           <t>Per-layer scoring</t>
         </is>
       </c>
-      <c r="C7" s="32" t="inlineStr">
+      <c r="C7" s="33" t="inlineStr">
         <is>
           <t>Each layer produces (points, has_data, reason). points are capped to prevent any single layer dominating; has_data is True when ANY field in the layer is populated (key bugfix: governance is True for all 4,410 DEF 14As scanned, not only those with PSU programs).</t>
         </is>
@@ -1819,7 +1822,7 @@
           <t>Coverage-normalised composite</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="C8" s="34" t="inlineStr">
         <is>
           <t>norm_score = raw_score × sqrt(7 / n_layers_present) for names with ≥3 layers. Names with 4 strong of 7 layers are not penalised vs names with 7 mediocre layers.</t>
         </is>
@@ -1834,7 +1837,7 @@
           <t>Per-pattern catalyst ranking</t>
         </is>
       </c>
-      <c r="C9" s="32" t="inlineStr">
+      <c r="C9" s="33" t="inlineStr">
         <is>
           <t>Top 10 in each of 18 catalyst patterns (forward $ hurdle, M&amp;A close, spin trigger, FDA milestone, etc.) — surfaces single-mandate leaders.</t>
         </is>
@@ -1849,7 +1852,7 @@
           <t>Archetype winners</t>
         </is>
       </c>
-      <c r="C10" s="33" t="inlineStr">
+      <c r="C10" s="34" t="inlineStr">
         <is>
           <t>57 PSU/governance/thesis buckets — single best representative of each archetype across the universe. Produces PSU_ARCHETYPES.md (38) + ASYMMETRIC_BY_ARCHETYPE.md (19).</t>
         </is>
@@ -1864,7 +1867,7 @@
           <t>Consensus meta-ranking</t>
         </is>
       </c>
-      <c r="C11" s="32" t="inlineStr">
+      <c r="C11" s="33" t="inlineStr">
         <is>
           <t>Each of 8 independent rankers + 2 archetype-winner markdowns contributes presence. n_screens = how many rankers surface the ticker. n_archetypes = how many buckets it wins. consensus_score = sum of rank-decay contributions.</t>
         </is>
@@ -1879,7 +1882,7 @@
           <t>Convergence test</t>
         </is>
       </c>
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C12" s="34" t="inlineStr">
         <is>
           <t>Name is convergent IFF n_screens ≥ 3 AND n_archetypes ≥ 1. Probability of 6-screen convergence by chance ≈ 2.4×10⁻¹⁰.</t>
         </is>
@@ -1894,7 +1897,7 @@
           <t>Robustness checks</t>
         </is>
       </c>
-      <c r="C13" s="32" t="inlineStr">
+      <c r="C13" s="33" t="inlineStr">
         <is>
           <t>Check 1: re-run after expanding yfinance from 1,885 to 2,132 (no change in convergent list). Check 2: governance bugfix expanded Tier-B coverage 2.8x (still no change). Convergent twelve is structurally informative, not data-dependent.</t>
         </is>
@@ -1909,7 +1912,7 @@
           <t>Caution layering</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C14" s="34" t="inlineStr">
         <is>
           <t>Eight red-flag classes scored from plan text: single-trigger CIC, repricing, retirement carveout, front-loaded grant, discretionary hurdle, aggregate-only metrics, plus structural. Convergence without direction; flag count modulates sizing.</t>
         </is>
@@ -1924,7 +1927,7 @@
           <t>Deployment / sizing</t>
         </is>
       </c>
-      <c r="C15" s="32" t="inlineStr">
+      <c r="C15" s="33" t="inlineStr">
         <is>
           <t>Concentrated (≥5%): clean convergent + ≥4 screens. Material (2-5%): 1-flag convergent or 4+ archetypes. Participation (0.5-2%): single-archetype or multi-flag. Basket (&lt;1% each): sub-archetype groups.</t>
         </is>
@@ -2073,7 +2076,7 @@
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 6.314</t>
+          <t>9 layers firing | cons 6.502</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">
@@ -2117,7 +2120,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.618</t>
+          <t>8 layers firing | cons 7.04</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr">
@@ -2134,34 +2137,36 @@
     <row r="7" ht="56" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>631</v>
+        <v>4180</v>
       </c>
       <c r="D7" s="19" t="n">
-        <v>15.29</v>
+        <v>14.42</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>14</v>
+        <v>1.34</v>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>spin_separation</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.354</t>
+          <t>8 layers firing | cons 6.79</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
@@ -2222,115 +2227,113 @@
     <row r="9" ht="56" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>NUS</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Nu Skin</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>244</v>
+        <v>631</v>
       </c>
       <c r="D9" s="19" t="n">
-        <v>5.02</v>
+        <v>15.29</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>0.31</v>
+        <v>0.76</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>asset_sale_named</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>Named asset-sale trigger + 5-metric clean per-share stack</t>
+          <t>8 layers firing | cons 5.326</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
-          <t>P/B 0.33 + buyback shrinking organically</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>see proxy_scan + buyback_verify</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
     <row r="10" ht="56" customHeight="1">
       <c r="A10" s="20" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>NUS</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>Nu Skin</t>
         </is>
       </c>
       <c r="C10" s="13" t="n">
-        <v>4180</v>
+        <v>244</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>14.42</v>
+        <v>5.02</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="F10" s="15" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>0.31</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>40</v>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>spin_separation</t>
+          <t>asset_sale_named</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.772</t>
+          <t>Named asset-sale trigger + 5-metric clean per-share stack</t>
         </is>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
-        </is>
-      </c>
-      <c r="J10" s="15" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>P/B 0.33 + buyback shrinking organically</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="11" ht="56" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>DXC Technology</t>
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>1043</v>
+        <v>1394</v>
       </c>
       <c r="D11" s="19" t="n">
-        <v>5.29</v>
+        <v>8.6</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.43</v>
+        <v>0.48</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
@@ -2339,56 +2342,56 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.49</t>
+          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
-        </is>
-      </c>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>IT services franchise; transformation signal in PSU</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="56" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Universal Display</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="C12" s="13" t="n">
-        <v>4158</v>
+        <v>1043</v>
       </c>
       <c r="D12" s="21" t="n">
-        <v>88.94</v>
+        <v>5.29</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>2.44</v>
+        <v>0.43</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>revenue_dollar_target</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
+          <t>7 layers firing | cons 5.532</t>
         </is>
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
-          <t>OLED IP moat</t>
+          <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
       <c r="J12" s="11" t="inlineStr">
@@ -2400,122 +2403,124 @@
     <row r="13" ht="56" customHeight="1">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>Universal Display</t>
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>124308</v>
+        <v>4158</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>151.78</v>
+        <v>88.94</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>3.63</v>
+        <v>2.44</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>revenue_dollar_target</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
+          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr">
         <is>
-          <t>Mega-cap recurring revenue base</t>
-        </is>
-      </c>
-      <c r="J13" s="16" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+          <t>OLED IP moat</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="14" ht="56" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>HDSN</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>Hudson Technologies</t>
         </is>
       </c>
       <c r="C14" s="13" t="n">
-        <v>7252</v>
+        <v>222</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>198.99</v>
+        <v>5.27</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>22</v>
+        <v>0.93</v>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>fda_phase_milestone</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.354</t>
+          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
         </is>
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
-        </is>
-      </c>
-      <c r="J14" s="15" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>Refrigerant reclaim regulatory moat</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="15" ht="56" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>9011</v>
+        <v>7252</v>
       </c>
       <c r="D15" s="19" t="n">
-        <v>176.03</v>
+        <v>198.99</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>4.58</v>
+        <v>6.4</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>fda_phase_milestone</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.352</t>
+          <t>7 layers firing | cons 5.338</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
@@ -2523,34 +2528,34 @@
           <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
-      <c r="J15" s="16" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
     <row r="16" ht="56" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>DXC</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>DXC Technology</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="C16" s="13" t="n">
-        <v>1394</v>
+        <v>9011</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>8.6</v>
+        <v>176.03</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>0.48</v>
+        <v>4.58</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>43</v>
+        <v>7</v>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
@@ -2559,12 +2564,12 @@
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
+          <t>7 layers firing | cons 5.336</t>
         </is>
       </c>
       <c r="I16" s="15" t="inlineStr">
         <is>
-          <t>IT services franchise; transformation signal in PSU</t>
+          <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
       <c r="J16" s="16" t="inlineStr">
@@ -2576,25 +2581,25 @@
     <row r="17" ht="56" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>PRGO</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>PRGO</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>1418</v>
+        <v>124308</v>
       </c>
       <c r="D17" s="19" t="n">
-        <v>10.25</v>
+        <v>151.78</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.57</v>
+        <v>3.63</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
@@ -2603,12 +2608,12 @@
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.112</t>
+          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
+          <t>Mega-cap recurring revenue base</t>
         </is>
       </c>
       <c r="J17" s="16" t="inlineStr">
@@ -2620,34 +2625,34 @@
     <row r="18" ht="56" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>GIII</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>GIII</t>
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>351</v>
+        <v>1467</v>
       </c>
       <c r="D18" s="21" t="n">
-        <v>16.44</v>
+        <v>34.77</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>ebitda_dollar_target</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.956</t>
+          <t>7 layers firing | cons 5.046</t>
         </is>
       </c>
       <c r="I18" s="15" t="inlineStr">
@@ -2664,25 +2669,25 @@
     <row r="19" ht="56" customHeight="1">
       <c r="A19" s="18" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>BLND</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>BLND</t>
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>1467</v>
+        <v>399</v>
       </c>
       <c r="D19" s="19" t="n">
-        <v>34.77</v>
+        <v>1.65</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>0.8</v>
+        <v>-7.3</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
@@ -2691,7 +2696,7 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.914</t>
+          <t>7 layers firing | cons 5.034</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
@@ -2699,34 +2704,34 @@
           <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
-      <c r="J19" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+      <c r="J19" s="11" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="20" ht="56" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>KMPR</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>Kemper</t>
         </is>
       </c>
       <c r="C20" s="13" t="n">
-        <v>862</v>
+        <v>1474</v>
       </c>
       <c r="D20" s="21" t="n">
-        <v>5.54</v>
+        <v>25.03</v>
       </c>
       <c r="E20" s="21" t="n">
-        <v>0.84</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
@@ -2735,88 +2740,88 @@
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.876</t>
+          <t>Anti-hedge/pledge + verified buyback EXECUTING (largest verified shrinkage)</t>
         </is>
       </c>
       <c r="I20" s="15" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
-        </is>
-      </c>
-      <c r="J20" s="16" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+          <t>Insurer at 0.54x book; $ repurchased = 1.85x NAV-accretive</t>
+        </is>
+      </c>
+      <c r="J20" s="15" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
     <row r="21" ht="56" customHeight="1">
       <c r="A21" s="18" t="inlineStr">
         <is>
-          <t>HDSN</t>
+          <t>PRGO</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Hudson Technologies</t>
+          <t>PRGO</t>
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>222</v>
+        <v>1418</v>
       </c>
       <c r="D21" s="19" t="n">
-        <v>5.27</v>
+        <v>10.25</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="F21" s="10" t="inlineStr">
+        <v>0.57</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="G21" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
+          <t>7 layers firing | cons 4.824</t>
         </is>
       </c>
       <c r="I21" s="10" t="inlineStr">
         <is>
-          <t>Refrigerant reclaim regulatory moat</t>
-        </is>
-      </c>
-      <c r="J21" s="11" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>see proxy_scan + buyback_verify</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
     <row r="22" ht="56" customHeight="1">
       <c r="A22" s="20" t="inlineStr">
         <is>
-          <t>KMPR</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>Kemper</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C22" s="13" t="n">
-        <v>1474</v>
+        <v>13781</v>
       </c>
       <c r="D22" s="21" t="n">
-        <v>25.03</v>
+        <v>121.36</v>
       </c>
       <c r="E22" s="21" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>27</v>
+        <v>2.85</v>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
@@ -2825,42 +2830,42 @@
       </c>
       <c r="H22" s="15" t="inlineStr">
         <is>
-          <t>Anti-hedge/pledge + verified buyback EXECUTING (largest verified shrinkage)</t>
+          <t>7 layers firing | cons 4.682</t>
         </is>
       </c>
       <c r="I22" s="15" t="inlineStr">
         <is>
-          <t>Insurer at 0.54x book; $ repurchased = 1.85x NAV-accretive</t>
-        </is>
-      </c>
-      <c r="J22" s="15" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>see proxy_scan + buyback_verify</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
     <row r="23" ht="56" customHeight="1">
       <c r="A23" s="18" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>Zoetis</t>
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>1074</v>
+        <v>32997</v>
       </c>
       <c r="D23" s="19" t="n">
-        <v>23.31</v>
+        <v>78.70999999999999</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>0.6899999999999999</v>
+        <v>10.04</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
@@ -2869,42 +2874,42 @@
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.406</t>
+          <t>F4 cluster + valuation + recent-incentive 60% drawdown</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
-        </is>
-      </c>
-      <c r="J23" s="11" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>Animal health franchise</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
     <row r="24" ht="56" customHeight="1">
       <c r="A24" s="20" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>CERT</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Zoetis</t>
+          <t>CERT</t>
         </is>
       </c>
       <c r="C24" s="13" t="n">
-        <v>32997</v>
+        <v>862</v>
       </c>
       <c r="D24" s="21" t="n">
-        <v>78.70999999999999</v>
+        <v>5.54</v>
       </c>
       <c r="E24" s="21" t="n">
-        <v>10.04</v>
+        <v>0.84</v>
       </c>
       <c r="F24" s="13" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
@@ -2913,17 +2918,17 @@
       </c>
       <c r="H24" s="15" t="inlineStr">
         <is>
-          <t>F4 cluster + valuation + recent-incentive 60% drawdown</t>
+          <t>7 layers firing | cons 4.524</t>
         </is>
       </c>
       <c r="I24" s="15" t="inlineStr">
         <is>
-          <t>Animal health franchise</t>
-        </is>
-      </c>
-      <c r="J24" s="15" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>see proxy_scan + buyback_verify</t>
+        </is>
+      </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
@@ -6665,7 +6670,7 @@
         <v>5.654</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
@@ -6733,7 +6738,7 @@
         <v>5.572</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
@@ -6767,7 +6772,7 @@
         <v>5.5</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
@@ -6801,7 +6806,7 @@
         <v>5.264</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
@@ -6835,7 +6840,7 @@
         <v>4.832</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
@@ -6869,7 +6874,7 @@
         <v>4.81</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
@@ -6903,7 +6908,7 @@
         <v>3.97</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
@@ -6971,7 +6976,7 @@
         <v>4.776</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
@@ -7005,7 +7010,7 @@
         <v>4.654</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
@@ -7039,7 +7044,7 @@
         <v>4.554</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
@@ -7073,7 +7078,7 @@
         <v>4.476</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>3</v>
+        <v>-4</v>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
@@ -7141,7 +7146,7 @@
         <v>4.424</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
@@ -7175,7 +7180,7 @@
         <v>4.414</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>-14</v>
+        <v>-12</v>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
@@ -7209,7 +7214,7 @@
         <v>4.27</v>
       </c>
       <c r="F22" s="13" t="n">
-        <v>-6</v>
+        <v>-11</v>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
@@ -7243,7 +7248,7 @@
         <v>4.086</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
@@ -7277,7 +7282,7 @@
         <v>3.942</v>
       </c>
       <c r="F24" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
@@ -7345,7 +7350,7 @@
         <v>3.566</v>
       </c>
       <c r="F26" s="13" t="n">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
@@ -7379,7 +7384,7 @@
         <v>3.42</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
@@ -7413,7 +7418,7 @@
         <v>3.386</v>
       </c>
       <c r="F28" s="13" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G28" s="15" t="inlineStr">
         <is>
@@ -7447,7 +7452,7 @@
         <v>3.226</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
@@ -7481,7 +7486,7 @@
         <v>2.866</v>
       </c>
       <c r="F30" s="13" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G30" s="15" t="inlineStr">
         <is>
@@ -7514,10 +7519,8 @@
       <c r="E31" s="19" t="n">
         <v>4.578</v>
       </c>
-      <c r="F31" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="F31" s="8" t="n">
+        <v>-1</v>
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
@@ -7550,8 +7553,10 @@
       <c r="E32" s="21" t="n">
         <v>4.524</v>
       </c>
-      <c r="F32" s="13" t="n">
-        <v>-2</v>
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G32" s="15" t="inlineStr">
         <is>
@@ -7584,8 +7589,8 @@
       <c r="E33" s="19" t="n">
         <v>4.506</v>
       </c>
-      <c r="F33" s="8" t="n">
-        <v>46</v>
+      <c r="F33" s="26" t="n">
+        <v>52</v>
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
@@ -7619,7 +7624,7 @@
         <v>4.366</v>
       </c>
       <c r="F34" s="13" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="G34" s="15" t="inlineStr">
         <is>
@@ -7759,7 +7764,7 @@
           <t>Repay Holdings Corporation</t>
         </is>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="D5" s="27" t="n">
         <v>68</v>
       </c>
       <c r="E5" s="8" t="n">
@@ -7773,7 +7778,7 @@
       <c r="G5" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="27" t="n">
+      <c r="H5" s="28" t="n">
         <v>44</v>
       </c>
       <c r="I5" s="19" t="n">
@@ -7799,7 +7804,7 @@
           <t>Gossamer Bio, Inc.</t>
         </is>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="D6" s="27" t="n">
         <v>61</v>
       </c>
       <c r="E6" s="13" t="n">
@@ -7813,7 +7818,7 @@
       <c r="G6" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="28" t="n">
+      <c r="H6" s="29" t="n">
         <v>96</v>
       </c>
       <c r="I6" s="21" t="n">
@@ -7839,7 +7844,7 @@
           <t>ZoomInfo Technologies Inc.</t>
         </is>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="27" t="n">
         <v>60</v>
       </c>
       <c r="E7" s="8" t="n">
@@ -7853,7 +7858,7 @@
       <c r="G7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="27" t="n">
+      <c r="H7" s="28" t="n">
         <v>78</v>
       </c>
       <c r="I7" s="19" t="n">
@@ -7879,7 +7884,7 @@
           <t>Goosehead Insurance, Inc.</t>
         </is>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="30" t="n">
         <v>53</v>
       </c>
       <c r="E8" s="13" t="n">
@@ -7893,7 +7898,7 @@
       <c r="G8" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="28" t="n">
+      <c r="H8" s="29" t="n">
         <v>70</v>
       </c>
       <c r="I8" s="21" t="n">
@@ -7919,7 +7924,7 @@
           <t>Guidewire Software, Inc.</t>
         </is>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="30" t="n">
         <v>53</v>
       </c>
       <c r="E9" s="8" t="n">
@@ -7933,7 +7938,7 @@
       <c r="G9" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="27" t="n">
+      <c r="H9" s="28" t="n">
         <v>60</v>
       </c>
       <c r="I9" s="19" t="n">
@@ -7959,7 +7964,7 @@
           <t>Comtech Telecommunications Corp</t>
         </is>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="30" t="n">
         <v>52</v>
       </c>
       <c r="E10" s="13" t="n">
@@ -7973,7 +7978,7 @@
       <c r="G10" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="28" t="n">
+      <c r="H10" s="29" t="n">
         <v>61</v>
       </c>
       <c r="I10" s="21" t="n">
@@ -7999,7 +8004,7 @@
           <t>BiomX Inc.</t>
         </is>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="30" t="n">
         <v>52</v>
       </c>
       <c r="E11" s="8" t="n">
@@ -8013,7 +8018,7 @@
       <c r="G11" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="27" t="n">
+      <c r="H11" s="28" t="n">
         <v>96</v>
       </c>
       <c r="I11" s="19" t="n">
@@ -8039,7 +8044,7 @@
           <t>ChargePoint Holdings, Inc.</t>
         </is>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="30" t="n">
         <v>52</v>
       </c>
       <c r="E12" s="13" t="n">
@@ -8053,7 +8058,7 @@
       <c r="G12" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="28" t="n">
+      <c r="H12" s="29" t="n">
         <v>49</v>
       </c>
       <c r="I12" s="21" t="n">
@@ -8079,7 +8084,7 @@
           <t>DXC Technology Company</t>
         </is>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="30" t="n">
         <v>52</v>
       </c>
       <c r="E13" s="8" t="n">
@@ -8093,7 +8098,7 @@
       <c r="G13" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="27" t="n">
+      <c r="H13" s="28" t="n">
         <v>48</v>
       </c>
       <c r="I13" s="19" t="n">
@@ -8119,7 +8124,7 @@
           <t>Processa Pharmaceuticals, Inc.</t>
         </is>
       </c>
-      <c r="D14" s="29" t="n">
+      <c r="D14" s="30" t="n">
         <v>51</v>
       </c>
       <c r="E14" s="13" t="n">
@@ -8133,7 +8138,7 @@
       <c r="G14" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="28" t="n">
+      <c r="H14" s="29" t="n">
         <v>86</v>
       </c>
       <c r="I14" s="21" t="n">
@@ -8159,7 +8164,7 @@
           <t>Peabody Energy Corporation</t>
         </is>
       </c>
-      <c r="D15" s="29" t="n">
+      <c r="D15" s="30" t="n">
         <v>51</v>
       </c>
       <c r="E15" s="8" t="n">
@@ -8173,7 +8178,7 @@
       <c r="G15" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="27" t="n">
+      <c r="H15" s="28" t="n">
         <v>36</v>
       </c>
       <c r="I15" s="19" t="n">
@@ -8199,7 +8204,7 @@
           <t>Ready Capital Corporation</t>
         </is>
       </c>
-      <c r="D16" s="29" t="n">
+      <c r="D16" s="30" t="n">
         <v>49</v>
       </c>
       <c r="E16" s="13" t="n">
@@ -8213,7 +8218,7 @@
       <c r="G16" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="28" t="n">
+      <c r="H16" s="29" t="n">
         <v>63</v>
       </c>
       <c r="I16" s="21" t="n">
@@ -8239,7 +8244,7 @@
           <t>Kingsway Corporation</t>
         </is>
       </c>
-      <c r="D17" s="29" t="n">
+      <c r="D17" s="30" t="n">
         <v>49</v>
       </c>
       <c r="E17" s="8" t="n">
@@ -8253,7 +8258,7 @@
       <c r="G17" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H17" s="27" t="n">
+      <c r="H17" s="28" t="n">
         <v>39</v>
       </c>
       <c r="I17" s="19" t="n">
@@ -8279,7 +8284,7 @@
           <t>Heron Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="D18" s="29" t="n">
+      <c r="D18" s="30" t="n">
         <v>48</v>
       </c>
       <c r="E18" s="13" t="n">
@@ -8293,7 +8298,7 @@
       <c r="G18" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="28" t="n">
+      <c r="H18" s="29" t="n">
         <v>82</v>
       </c>
       <c r="I18" s="21" t="n">
@@ -8319,7 +8324,7 @@
           <t>Standard BioTools Inc.</t>
         </is>
       </c>
-      <c r="D19" s="29" t="n">
+      <c r="D19" s="30" t="n">
         <v>48</v>
       </c>
       <c r="E19" s="8" t="n">
@@ -8333,7 +8338,7 @@
       <c r="G19" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H19" s="27" t="n">
+      <c r="H19" s="28" t="n">
         <v>52</v>
       </c>
       <c r="I19" s="19" t="n">
@@ -8359,7 +8364,7 @@
           <t>InspireMD Inc.</t>
         </is>
       </c>
-      <c r="D20" s="29" t="n">
+      <c r="D20" s="30" t="n">
         <v>47</v>
       </c>
       <c r="E20" s="13" t="n">
@@ -8373,7 +8378,7 @@
       <c r="G20" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="28" t="n">
+      <c r="H20" s="29" t="n">
         <v>76</v>
       </c>
       <c r="I20" s="21" t="n">
@@ -8399,7 +8404,7 @@
           <t>Rein Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="D21" s="29" t="n">
+      <c r="D21" s="30" t="n">
         <v>46</v>
       </c>
       <c r="E21" s="8" t="n">
@@ -8413,7 +8418,7 @@
       <c r="G21" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="27" t="n">
+      <c r="H21" s="28" t="n">
         <v>58</v>
       </c>
       <c r="I21" s="19" t="n">
@@ -8439,7 +8444,7 @@
           <t>Booz Allen Hamilton Holding Cor</t>
         </is>
       </c>
-      <c r="D22" s="29" t="n">
+      <c r="D22" s="30" t="n">
         <v>46</v>
       </c>
       <c r="E22" s="13" t="n">
@@ -8453,7 +8458,7 @@
       <c r="G22" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="28" t="n">
+      <c r="H22" s="29" t="n">
         <v>45</v>
       </c>
       <c r="I22" s="21" t="n">
@@ -8479,7 +8484,7 @@
           <t>VolitionRX Limited</t>
         </is>
       </c>
-      <c r="D23" s="29" t="n">
+      <c r="D23" s="30" t="n">
         <v>45</v>
       </c>
       <c r="E23" s="8" t="n">
@@ -8493,7 +8498,7 @@
       <c r="G23" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="27" t="n">
+      <c r="H23" s="28" t="n">
         <v>92</v>
       </c>
       <c r="I23" s="19" t="n">
@@ -8519,7 +8524,7 @@
           <t>Total Return Securities Fund</t>
         </is>
       </c>
-      <c r="D24" s="29" t="n">
+      <c r="D24" s="30" t="n">
         <v>44</v>
       </c>
       <c r="E24" s="13" t="n">
@@ -8533,7 +8538,7 @@
       <c r="G24" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H24" s="28" t="n">
+      <c r="H24" s="29" t="n">
         <v>8</v>
       </c>
       <c r="I24" s="21" t="n">
@@ -8559,7 +8564,7 @@
           <t>Fox Corporation</t>
         </is>
       </c>
-      <c r="D25" s="29" t="n">
+      <c r="D25" s="30" t="n">
         <v>44</v>
       </c>
       <c r="E25" s="8" t="n">
@@ -8573,7 +8578,7 @@
       <c r="G25" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H25" s="27" t="n">
+      <c r="H25" s="28" t="n">
         <v>31</v>
       </c>
       <c r="I25" s="19" t="n">
@@ -8599,7 +8604,7 @@
           <t>Outlook Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="D26" s="29" t="n">
+      <c r="D26" s="30" t="n">
         <v>44</v>
       </c>
       <c r="E26" s="13" t="n">
@@ -8613,7 +8618,7 @@
       <c r="G26" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="H26" s="28" t="n">
+      <c r="H26" s="29" t="n">
         <v>53</v>
       </c>
       <c r="I26" s="21" t="n">
@@ -8639,7 +8644,7 @@
           <t>My Size, Inc.</t>
         </is>
       </c>
-      <c r="D27" s="29" t="n">
+      <c r="D27" s="30" t="n">
         <v>43</v>
       </c>
       <c r="E27" s="8" t="n">
@@ -8653,7 +8658,7 @@
       <c r="G27" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="27" t="n">
+      <c r="H27" s="28" t="n">
         <v>72</v>
       </c>
       <c r="I27" s="19" t="n">
@@ -8679,7 +8684,7 @@
           <t>Purple Innovation, Inc.</t>
         </is>
       </c>
-      <c r="D28" s="29" t="n">
+      <c r="D28" s="30" t="n">
         <v>43</v>
       </c>
       <c r="E28" s="13" t="n">
@@ -8693,7 +8698,7 @@
       <c r="G28" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="28" t="n">
+      <c r="H28" s="29" t="n">
         <v>66</v>
       </c>
       <c r="I28" s="21" t="n">
@@ -8719,7 +8724,7 @@
           <t>Cosmos Health Inc.</t>
         </is>
       </c>
-      <c r="D29" s="29" t="n">
+      <c r="D29" s="30" t="n">
         <v>43</v>
       </c>
       <c r="E29" s="8" t="n">
@@ -8733,7 +8738,7 @@
       <c r="G29" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H29" s="27" t="n">
+      <c r="H29" s="28" t="n">
         <v>84</v>
       </c>
       <c r="I29" s="19" t="n">
@@ -8759,7 +8764,7 @@
           <t>Power Solutions International,</t>
         </is>
       </c>
-      <c r="D30" s="29" t="n">
+      <c r="D30" s="30" t="n">
         <v>43</v>
       </c>
       <c r="E30" s="13" t="n">
@@ -8773,7 +8778,7 @@
       <c r="G30" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H30" s="28" t="n">
+      <c r="H30" s="29" t="n">
         <v>67</v>
       </c>
       <c r="I30" s="21" t="n">
@@ -8799,7 +8804,7 @@
           <t>NexGel, Inc</t>
         </is>
       </c>
-      <c r="D31" s="29" t="n">
+      <c r="D31" s="30" t="n">
         <v>43</v>
       </c>
       <c r="E31" s="8" t="n">
@@ -8813,7 +8818,7 @@
       <c r="G31" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H31" s="27" t="n">
+      <c r="H31" s="28" t="n">
         <v>80</v>
       </c>
       <c r="I31" s="19" t="n">
@@ -8839,7 +8844,7 @@
           <t>Salesforce, Inc.</t>
         </is>
       </c>
-      <c r="D32" s="29" t="n">
+      <c r="D32" s="30" t="n">
         <v>42</v>
       </c>
       <c r="E32" s="13" t="n">
@@ -8853,7 +8858,7 @@
       <c r="G32" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="H32" s="28" t="n">
+      <c r="H32" s="29" t="n">
         <v>45</v>
       </c>
       <c r="I32" s="21" t="n">
@@ -8879,7 +8884,7 @@
           <t>Vitesse Energy, Inc.</t>
         </is>
       </c>
-      <c r="D33" s="29" t="n">
+      <c r="D33" s="30" t="n">
         <v>42</v>
       </c>
       <c r="E33" s="8" t="n">
@@ -8893,7 +8898,7 @@
       <c r="G33" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H33" s="27" t="n">
+      <c r="H33" s="28" t="n">
         <v>41</v>
       </c>
       <c r="I33" s="19" t="n">
@@ -8919,7 +8924,7 @@
           <t>Krispy Kreme, Inc.</t>
         </is>
       </c>
-      <c r="D34" s="29" t="n">
+      <c r="D34" s="30" t="n">
         <v>42</v>
       </c>
       <c r="E34" s="13" t="n">
@@ -8933,7 +8938,7 @@
       <c r="G34" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H34" s="28" t="n">
+      <c r="H34" s="29" t="n">
         <v>37</v>
       </c>
       <c r="I34" s="21" t="n">
@@ -8959,7 +8964,7 @@
           <t>Nerdy Inc.</t>
         </is>
       </c>
-      <c r="D35" s="29" t="n">
+      <c r="D35" s="30" t="n">
         <v>41</v>
       </c>
       <c r="E35" s="8" t="n">
@@ -8973,7 +8978,7 @@
       <c r="G35" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H35" s="27" t="n">
+      <c r="H35" s="28" t="n">
         <v>51</v>
       </c>
       <c r="I35" s="19" t="n">
@@ -8999,7 +9004,7 @@
           <t>Artiva Biotherapeutics, Inc.</t>
         </is>
       </c>
-      <c r="D36" s="29" t="n">
+      <c r="D36" s="30" t="n">
         <v>41</v>
       </c>
       <c r="E36" s="13" t="n">
@@ -9013,7 +9018,7 @@
       <c r="G36" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H36" s="28" t="n">
+      <c r="H36" s="29" t="n">
         <v>49</v>
       </c>
       <c r="I36" s="21" t="n">
@@ -9039,7 +9044,7 @@
           <t>STERIS plc (Ireland)</t>
         </is>
       </c>
-      <c r="D37" s="29" t="n">
+      <c r="D37" s="30" t="n">
         <v>41</v>
       </c>
       <c r="E37" s="8" t="n">
@@ -9053,7 +9058,7 @@
       <c r="G37" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H37" s="27" t="n">
+      <c r="H37" s="28" t="n">
         <v>25</v>
       </c>
       <c r="I37" s="19" t="n">
@@ -9079,7 +9084,7 @@
           <t>Rubrik, Inc.</t>
         </is>
       </c>
-      <c r="D38" s="29" t="n">
+      <c r="D38" s="30" t="n">
         <v>41</v>
       </c>
       <c r="E38" s="13" t="n">
@@ -9093,7 +9098,7 @@
       <c r="G38" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H38" s="28" t="n">
+      <c r="H38" s="29" t="n">
         <v>30</v>
       </c>
       <c r="I38" s="21" t="n">
@@ -9119,7 +9124,7 @@
           <t>Medline Inc.</t>
         </is>
       </c>
-      <c r="D39" s="29" t="n">
+      <c r="D39" s="30" t="n">
         <v>40</v>
       </c>
       <c r="E39" s="8" t="n">
@@ -9133,7 +9138,7 @@
       <c r="G39" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H39" s="27" t="n">
+      <c r="H39" s="28" t="n">
         <v>29</v>
       </c>
       <c r="I39" s="19" t="n">
@@ -9159,7 +9164,7 @@
           <t>Toro Corp.</t>
         </is>
       </c>
-      <c r="D40" s="29" t="n">
+      <c r="D40" s="30" t="n">
         <v>40</v>
       </c>
       <c r="E40" s="13" t="n">
@@ -9173,7 +9178,7 @@
       <c r="G40" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H40" s="28" t="n">
+      <c r="H40" s="29" t="n">
         <v>40</v>
       </c>
       <c r="I40" s="21" t="n">
@@ -9199,7 +9204,7 @@
           <t>CuriosityStream Inc.</t>
         </is>
       </c>
-      <c r="D41" s="29" t="n">
+      <c r="D41" s="30" t="n">
         <v>40</v>
       </c>
       <c r="E41" s="8" t="n">
@@ -9213,7 +9218,7 @@
       <c r="G41" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H41" s="27" t="n">
+      <c r="H41" s="28" t="n">
         <v>57</v>
       </c>
       <c r="I41" s="19" t="n">
@@ -9239,7 +9244,7 @@
           <t>Health Catalyst, Inc</t>
         </is>
       </c>
-      <c r="D42" s="29" t="n">
+      <c r="D42" s="30" t="n">
         <v>40</v>
       </c>
       <c r="E42" s="13" t="n">
@@ -9253,7 +9258,7 @@
       <c r="G42" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H42" s="28" t="n">
+      <c r="H42" s="29" t="n">
         <v>55</v>
       </c>
       <c r="I42" s="21" t="n">
@@ -9293,7 +9298,7 @@
       <c r="G43" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H43" s="27" t="n">
+      <c r="H43" s="28" t="n">
         <v>87</v>
       </c>
       <c r="I43" s="19" t="n">
@@ -9333,7 +9338,7 @@
       <c r="G44" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="H44" s="28" t="n">
+      <c r="H44" s="29" t="n">
         <v>63</v>
       </c>
       <c r="I44" s="21" t="n">
@@ -9472,7 +9477,7 @@
           <t>Jet.AI Inc.</t>
         </is>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D5" s="30" t="n">
         <v>43</v>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -9514,7 +9519,7 @@
           <t>BEYOND MEAT, INC.</t>
         </is>
       </c>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="30" t="n">
         <v>35</v>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -9556,7 +9561,7 @@
           <t>COMTECH TELECOMMUNICATIONS CORP</t>
         </is>
       </c>
-      <c r="D7" s="29" t="n">
+      <c r="D7" s="30" t="n">
         <v>35</v>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -9598,7 +9603,7 @@
           <t>FISERV INC</t>
         </is>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="30" t="n">
         <v>35</v>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -9640,7 +9645,7 @@
           <t>BTCS Inc.</t>
         </is>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="30" t="n">
         <v>35</v>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -9682,7 +9687,7 @@
           <t>HERON THERAPEUTICS, INC. /DE/</t>
         </is>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="30" t="n">
         <v>35</v>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -9724,7 +9729,7 @@
           <t>WW INTERNATIONAL, INC.</t>
         </is>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="30" t="n">
         <v>33</v>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -11192,7 +11197,7 @@
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>Highest PSU forensic core</t>
         </is>
@@ -11462,7 +11467,7 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Highest governance score</t>
         </is>
@@ -11732,7 +11737,7 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="30" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
         <is>
           <t>Deepest P/B floor (&lt;0.5x book)</t>
         </is>
@@ -12002,7 +12007,7 @@
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="30" t="inlineStr">
+      <c r="A40" s="31" t="inlineStr">
         <is>
           <t>Cheapest EV/EBITDA (&lt;6x)</t>
         </is>
@@ -12272,7 +12277,7 @@
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="30" t="inlineStr">
+      <c r="A52" s="31" t="inlineStr">
         <is>
           <t>Lowest trailing P/E (&lt;8x, positive)</t>
         </is>
@@ -12542,7 +12547,7 @@
       </c>
     </row>
     <row r="64" ht="22" customHeight="1">
-      <c r="A64" s="30" t="inlineStr">
+      <c r="A64" s="31" t="inlineStr">
         <is>
           <t>Largest verified buyback shrinkage</t>
         </is>
@@ -12812,7 +12817,7 @@
       </c>
     </row>
     <row r="76" ht="22" customHeight="1">
-      <c r="A76" s="30" t="inlineStr">
+      <c r="A76" s="31" t="inlineStr">
         <is>
           <t>Highest 10b5-1 termination signed score</t>
         </is>
@@ -13082,7 +13087,7 @@
       </c>
     </row>
     <row r="88" ht="22" customHeight="1">
-      <c r="A88" s="30" t="inlineStr">
+      <c r="A88" s="31" t="inlineStr">
         <is>
           <t>Largest insider Form 4 dollar cluster</t>
         </is>
@@ -13352,7 +13357,7 @@
       </c>
     </row>
     <row r="100" ht="22" customHeight="1">
-      <c r="A100" s="30" t="inlineStr">
+      <c r="A100" s="31" t="inlineStr">
         <is>
           <t>Live tender / 13E-3 events</t>
         </is>

</xml_diff>

<commit_message>
Refresh all deliverables via rebuild_all.sh (post ticker-gate)
Full derived-only regeneration through the one-command runner:
consensus (val + noval), layer correlation, freshness, systematic
rankings, and the 14-tab workbook. Universe clean at 6,166.

Current top of universe (30 layers):
   1. FOUR  9L    (uniquely top)
   2. EPAM  8L    6. PAR   8L
   3. GPGI  8L    7. HUBS  7L
   4. ADT   8L    8. OLED  7L
   5. CRM   8L    9. SBET  7L
                 10. NUS   7L   11. PRGO 7L   12. POOL 7L
</commit_message>
<xml_diff>
--- a/MOST_ASYMMETRIC.xlsx
+++ b/MOST_ASYMMETRIC.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -186,6 +186,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -939,7 +942,7 @@
           <t>Jet.AI Inc.</t>
         </is>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="20" t="n">
         <v>43</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -981,7 +984,7 @@
           <t>BEYOND MEAT, INC.</t>
         </is>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="20" t="n">
         <v>35</v>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -1023,7 +1026,7 @@
           <t>COMTECH TELECOMMUNICATIONS CORP</t>
         </is>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="20" t="n">
         <v>35</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1065,7 +1068,7 @@
           <t>FISERV INC</t>
         </is>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="20" t="n">
         <v>35</v>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -1107,7 +1110,7 @@
           <t>BTCS Inc.</t>
         </is>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="20" t="n">
         <v>35</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1149,7 +1152,7 @@
           <t>HERON THERAPEUTICS, INC. /DE/</t>
         </is>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="20" t="n">
         <v>35</v>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -1191,7 +1194,7 @@
           <t>WW INTERNATIONAL, INC.</t>
         </is>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="20" t="n">
         <v>33</v>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -2662,14 +2665,14 @@
     </row>
     <row r="3" ht="8" customHeight="1"/>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>Highest PSU forensic core</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>What it measures: depth + rigor of the PSU plan</t>
         </is>
@@ -2932,14 +2935,14 @@
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>Highest governance score</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>What it measures: clawback + anti-hedge + vesting + ownership multiple</t>
         </is>
@@ -3202,14 +3205,14 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>Deepest P/B floor (&lt;0.5x book)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="inlineStr">
+      <c r="A29" s="24" t="inlineStr">
         <is>
           <t>What it measures: hard balance-sheet value floor</t>
         </is>
@@ -3472,14 +3475,14 @@
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="22" t="inlineStr">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>Cheapest EV/EBITDA (&lt;6x)</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="23" t="inlineStr">
+      <c r="A41" s="24" t="inlineStr">
         <is>
           <t>What it measures: enterprise-value to earnings power</t>
         </is>
@@ -3742,14 +3745,14 @@
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="22" t="inlineStr">
+      <c r="A52" s="23" t="inlineStr">
         <is>
           <t>Lowest trailing P/E (&lt;8x, positive)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="23" t="inlineStr">
+      <c r="A53" s="24" t="inlineStr">
         <is>
           <t>What it measures: earnings yield</t>
         </is>
@@ -4012,14 +4015,14 @@
       </c>
     </row>
     <row r="64" ht="22" customHeight="1">
-      <c r="A64" s="22" t="inlineStr">
+      <c r="A64" s="23" t="inlineStr">
         <is>
           <t>Largest verified buyback shrinkage</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="23" t="inlineStr">
+      <c r="A65" s="24" t="inlineStr">
         <is>
           <t>What it measures: actual supply curve compression</t>
         </is>
@@ -4282,14 +4285,14 @@
       </c>
     </row>
     <row r="76" ht="22" customHeight="1">
-      <c r="A76" s="22" t="inlineStr">
+      <c r="A76" s="23" t="inlineStr">
         <is>
           <t>Highest 10b5-1 termination signed score</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="23" t="inlineStr">
+      <c r="A77" s="24" t="inlineStr">
         <is>
           <t>What it measures: insider walked back scheduled selling</t>
         </is>
@@ -4552,14 +4555,14 @@
       </c>
     </row>
     <row r="88" ht="22" customHeight="1">
-      <c r="A88" s="22" t="inlineStr">
+      <c r="A88" s="23" t="inlineStr">
         <is>
           <t>Largest insider Form 4 dollar cluster</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="23" t="inlineStr">
+      <c r="A89" s="24" t="inlineStr">
         <is>
           <t>What it measures: insider conviction in dollars</t>
         </is>
@@ -4822,14 +4825,14 @@
       </c>
     </row>
     <row r="100" ht="22" customHeight="1">
-      <c r="A100" s="22" t="inlineStr">
+      <c r="A100" s="23" t="inlineStr">
         <is>
           <t>Live tender / 13E-3 events</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="23" t="inlineStr">
+      <c r="A101" s="24" t="inlineStr">
         <is>
           <t>What it measures: mechanical bid as floor</t>
         </is>
@@ -5298,7 +5301,7 @@
         </is>
       </c>
       <c r="C9" s="16" t="n">
-        <v>0.67</v>
+        <v>0.667</v>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
@@ -5378,7 +5381,7 @@
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>0.58</v>
+        <v>0.581</v>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
@@ -5578,7 +5581,7 @@
         </is>
       </c>
       <c r="C23" s="16" t="n">
-        <v>0.341</v>
+        <v>0.34</v>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
@@ -5658,7 +5661,7 @@
         </is>
       </c>
       <c r="C27" s="16" t="n">
-        <v>0.272</v>
+        <v>0.274</v>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
@@ -5804,12 +5807,12 @@
       <c r="B5" s="16" t="n">
         <v>4410</v>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="21" t="n">
         <v>71.54445165476963</v>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>15d</t>
+          <t>19d</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -5832,12 +5835,12 @@
       <c r="B6" s="17" t="n">
         <v>4410</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="22" t="n">
         <v>71.54445165476963</v>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>15d</t>
+          <t>19d</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -5860,12 +5863,12 @@
       <c r="B7" s="16" t="n">
         <v>6164</v>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="21" t="n">
         <v>100</v>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>15d</t>
+          <t>19d</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -5888,12 +5891,12 @@
       <c r="B8" s="17" t="n">
         <v>6164</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="22" t="n">
         <v>100</v>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>16d</t>
+          <t>20d</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -5916,12 +5919,12 @@
       <c r="B9" s="16" t="n">
         <v>2935</v>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="21" t="n">
         <v>47.61518494484101</v>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>16d</t>
+          <t>20d</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -5944,12 +5947,12 @@
       <c r="B10" s="17" t="n">
         <v>2807</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="22" t="n">
         <v>45.53861129136924</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>7d</t>
+          <t>11d</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -5972,12 +5975,12 @@
       <c r="B11" s="16" t="n">
         <v>1221</v>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="21" t="n">
         <v>19.80856586632057</v>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>9d</t>
+          <t>13d</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -6000,12 +6003,12 @@
       <c r="B12" s="17" t="n">
         <v>346</v>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C12" s="22" t="n">
         <v>5.613238157040882</v>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>25d</t>
+          <t>30d</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -6028,12 +6031,12 @@
       <c r="B13" s="16" t="n">
         <v>346</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="21" t="n">
         <v>5.613238157040882</v>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>5d</t>
+          <t>10d</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -6056,7 +6059,7 @@
       <c r="B14" s="17" t="n">
         <v>164</v>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="22" t="n">
         <v>2.660609993510707</v>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -6084,12 +6087,12 @@
       <c r="B15" s="16" t="n">
         <v>260</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="21" t="n">
         <v>4.218040233614536</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>4d</t>
+          <t>8d</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -6112,12 +6115,12 @@
       <c r="B16" s="17" t="n">
         <v>1982</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="22" t="n">
         <v>32.15444516547696</v>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>5d</t>
+          <t>9d</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -6140,12 +6143,12 @@
       <c r="B17" s="16" t="n">
         <v>1180</v>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="21" t="n">
         <v>19.14341336794289</v>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>5d</t>
+          <t>9d</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -6168,7 +6171,7 @@
       <c r="B18" s="17" t="n">
         <v>1167</v>
       </c>
-      <c r="C18" s="21" t="n">
+      <c r="C18" s="22" t="n">
         <v>18.93251135626216</v>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -6196,7 +6199,7 @@
       <c r="B19" s="16" t="n">
         <v>46</v>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="21" t="n">
         <v>0.7462686567164178</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -6224,7 +6227,7 @@
       <c r="B20" s="17" t="n">
         <v>209</v>
       </c>
-      <c r="C20" s="21" t="n">
+      <c r="C20" s="22" t="n">
         <v>3.390655418559377</v>
       </c>
       <c r="D20" s="10" t="inlineStr">
@@ -6252,7 +6255,7 @@
       <c r="B21" s="16" t="n">
         <v>71</v>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="21" t="n">
         <v>1.151849448410123</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -6280,12 +6283,12 @@
       <c r="B22" s="17" t="n">
         <v>25</v>
       </c>
-      <c r="C22" s="21" t="n">
+      <c r="C22" s="22" t="n">
         <v>0.4055807916937054</v>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>4d</t>
+          <t>8d</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -6308,7 +6311,7 @@
       <c r="B23" s="16" t="n">
         <v>89</v>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="21" t="n">
         <v>1.443867618429591</v>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -6420,7 +6423,7 @@
         <v>4</v>
       </c>
       <c r="B32" s="16" t="n">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
@@ -6433,7 +6436,7 @@
         <v>3</v>
       </c>
       <c r="B33" s="17" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
@@ -6446,7 +6449,7 @@
         <v>2</v>
       </c>
       <c r="B34" s="16" t="n">
-        <v>673</v>
+        <v>667</v>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
@@ -6459,7 +6462,7 @@
         <v>1</v>
       </c>
       <c r="B35" s="17" t="n">
-        <v>1105</v>
+        <v>1111</v>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
@@ -6553,7 +6556,7 @@
           <t>Universe construction</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>6,164 US-listed common tickers from cancel_10b5_1.json — authoritative NYSE/Nasdaq/AMEX/CBOE set. Foreign names (JP/KR/UK) live in a separate tab and universe.</t>
         </is>
@@ -6568,7 +6571,7 @@
           <t>Layer ingestion</t>
         </is>
       </c>
-      <c r="C6" s="25" t="inlineStr">
+      <c r="C6" s="26" t="inlineStr">
         <is>
           <t>30 additive scoring layers ingested per ticker, spanning PSU forensics, governance, valuation, verified buybacks, tender mechanics, 10b5-1 direction, Form 4 (raw + Cohen-Malloy opportunistic), Form 144, quarterly 10-Q, NCAV, Voss CIC, post-Ch11, internalization, bumpitrage, spinoff timing, Arquitos, Coval-Stafford proxy + real N-PORT, backstopped rights, FDIC dark banks, activist letters, 13F-delta, biotech PDUFA, and financial-sector primary.</t>
         </is>
@@ -6583,7 +6586,7 @@
           <t>Additive discipline</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Every layer ADDS to the composite; none modifies another's score. New legs append fields; existing weights never change. This is enforced and audited (verify_universe_methodology.py).</t>
         </is>
@@ -6598,7 +6601,7 @@
           <t>Coverage-normalised composite</t>
         </is>
       </c>
-      <c r="C8" s="25" t="inlineStr">
+      <c r="C8" s="26" t="inlineStr">
         <is>
           <t>Sparse-coverage names are not penalised for missing layers; the norm score rescales by sqrt(n_total/n_present) so a name strong on few layers competes with a name mediocre on many.</t>
         </is>
@@ -6613,7 +6616,7 @@
           <t>Per-pattern catalyst ranking</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>Top names in each catalyst pattern (forward $ hurdle, M&amp;A close, spin trigger, FDA/PDUFA, post-Ch11, asset sale, etc.) — surfaces single-mandate leaders (see Single-Measure tab).</t>
         </is>
@@ -6628,7 +6631,7 @@
           <t>Archetype winners</t>
         </is>
       </c>
-      <c r="C10" s="25" t="inlineStr">
+      <c r="C10" s="26" t="inlineStr">
         <is>
           <t>57 PSU/governance/thesis buckets — single best representative of each archetype across the universe (PSU_ARCHETYPES.md 38 + ASYMMETRIC_BY_ARCHETYPE.md 19).</t>
         </is>
@@ -6643,7 +6646,7 @@
           <t>Consensus meta-ranking</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>n_layers_firing = how many of the 30 independent layers produce a non-zero score for the ticker. consensus_score = sum of per-layer rank-decay contributions across the universe.</t>
         </is>
@@ -6658,7 +6661,7 @@
           <t>Layer independence</t>
         </is>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>Pairwise Spearman correlation (layer_correlation_pairs.csv) collapses 30 raw layers to ~21 effective-independent at rho&gt;0.6. Three correlated clusters: PSU+Voss, tender family, F4+opportunistic. 'Fires 9 layers' ≈ 7-8 true confirmations.</t>
         </is>
@@ -6673,7 +6676,7 @@
           <t>Freshness weighting</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>layer_freshness.json records each layer's data age. Most layers are &lt;14 days old. An optional age-decay multiplier (opt-in) can down-weight stale layers; current build reports age without auto-decaying.</t>
         </is>
@@ -6688,7 +6691,7 @@
           <t>Caution layering</t>
         </is>
       </c>
-      <c r="C14" s="25" t="inlineStr">
+      <c r="C14" s="26" t="inlineStr">
         <is>
           <t>Eight red-flag classes from plan text: single-trigger CIC, repricing, retirement carveout, front-loaded grant, discretionary hurdle, aggregate-only metrics, plus structural. Convergence without direction; flag count modulates sizing.</t>
         </is>
@@ -6703,7 +6706,7 @@
           <t>Deployment / sizing</t>
         </is>
       </c>
-      <c r="C15" s="24" t="inlineStr">
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t>Concentrated (≥5%): clean high-layer-count names. Material (2-5%): strong but 1-2 flags. Participation (0.5-2%): single-leg or multi-flag. Basket (&lt;1% each): sub-archetype groups, Cohen-Malloy stack, R2000-boundary, NOL shells, foreign.</t>
         </is>
@@ -6718,7 +6721,7 @@
           <t>Honest limitations</t>
         </is>
       </c>
-      <c r="C16" s="25" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>No realized-return backtest yet (AUDIT.md S1.1) — the composite is a structurally-sound pattern-recognition system, not yet validated alpha. Cohen-Malloy needs deeper Form 4 history. Coval-Stafford proxy supplements but does not replace the N-PORT real signal. See AUDIT.md for the full ledger.</t>
         </is>
@@ -6938,7 +6941,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 6.088</t>
+          <t>9 layers firing | cons 6.154</t>
         </is>
       </c>
     </row>
@@ -6948,22 +6951,22 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>EPAM</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>GPGI</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>EPAM</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.768</t>
+          <t>8 layers firing | cons 6.876</t>
         </is>
       </c>
     </row>
@@ -6973,22 +6976,22 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>EPAM</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>EPAM</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+          <t>GPGI</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.626</t>
+          <t>8 layers firing | cons 6.574</t>
         </is>
       </c>
     </row>
@@ -6998,22 +7001,22 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>ADT</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>ADT Inc</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Participation 1-2%</t>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
+          <t>Heaviest PSU%LTI in universe (90%) + verified -7.3% shrinkage</t>
         </is>
       </c>
     </row>
@@ -7023,22 +7026,22 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>ADT Inc</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>Heaviest PSU%LTI in universe (90%) + verified -7.3% shrinkage</t>
+          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7066,7 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.336</t>
+          <t>8 layers firing | cons 5.704</t>
         </is>
       </c>
     </row>
@@ -7088,7 +7091,7 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.812</t>
+          <t>7 layers firing | cons 5.802</t>
         </is>
       </c>
     </row>
@@ -7098,12 +7101,12 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>Universal Display</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -7113,7 +7116,7 @@
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.706</t>
+          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
         </is>
       </c>
     </row>
@@ -7123,22 +7126,22 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>DXC</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>DXC Technology</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Participation 1-2%</t>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
+          <t>7 layers firing | cons 5.522</t>
         </is>
       </c>
     </row>
@@ -7148,22 +7151,22 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>NUS</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>GIII</t>
-        </is>
-      </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>Nu Skin</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.398</t>
+          <t>Named asset-sale trigger + 5-metric clean per-share stack</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7191,7 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.328</t>
+          <t>7 layers firing | cons 5.332</t>
         </is>
       </c>
     </row>
@@ -7198,22 +7201,22 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Universal Display</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>POOL</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
+          <t>7 layers firing | cons 5.26</t>
         </is>
       </c>
     </row>
@@ -7223,22 +7226,22 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>NUS</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Nu Skin</t>
+          <t>DXC Technology</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Named asset-sale trigger + 5-metric clean per-share stack</t>
+          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
         </is>
       </c>
     </row>
@@ -7248,22 +7251,22 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>CERT</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>POOL</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>CERT</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.87</t>
+          <t>7 layers firing | cons 5.002</t>
         </is>
       </c>
     </row>
@@ -7288,7 +7291,7 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.85</t>
+          <t>7 layers firing | cons 4.94</t>
         </is>
       </c>
     </row>
@@ -7323,22 +7326,22 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>HDSN</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Hudson Technologies</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>Zoetis</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
+          <t>F4 cluster + valuation + recent-incentive 60% drawdown</t>
         </is>
       </c>
     </row>
@@ -7348,22 +7351,22 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>HDSN</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>Hudson Technologies</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Participation 1-2%</t>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.64</t>
+          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
         </is>
       </c>
     </row>
@@ -7373,22 +7376,22 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.452</t>
+          <t>7 layers firing | cons 4.658</t>
         </is>
       </c>
     </row>
@@ -7398,12 +7401,12 @@
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>GIII</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>GIII</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
@@ -7413,7 +7416,7 @@
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.45</t>
+          <t>7 layers firing | cons 4.656</t>
         </is>
       </c>
     </row>
@@ -7591,7 +7594,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 6.088</t>
+          <t>9 layers firing | cons 6.154</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -7608,36 +7611,34 @@
     <row r="6" ht="56" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>EPAM</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>EPAM</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>4180</v>
+        <v>4004</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>14.42</v>
+        <v>76.64</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
+        <v>1.18</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>spin_separation</t>
-        </is>
-      </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.768</t>
+          <t>8 layers firing | cons 6.876</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
@@ -7645,43 +7646,45 @@
           <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
-      <c r="J6" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
     <row r="7" ht="56" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>EPAM</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>EPAM</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>4004</v>
+        <v>4180</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>76.64</v>
+        <v>14.42</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>14</v>
+        <v>1.34</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>spin_separation</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.626</t>
+          <t>8 layers firing | cons 6.574</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
@@ -7689,34 +7692,34 @@
           <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
     <row r="8" ht="56" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>ADT</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>ADT Inc</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>124308</v>
+        <v>5004</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>151.78</v>
+        <v>6.58</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>3.63</v>
+        <v>1.38</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
@@ -7725,42 +7728,42 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
+          <t>Heaviest PSU%LTI in universe (90%) + verified -7.3% shrinkage</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>Mega-cap recurring revenue base</t>
+          <t>Recurring monitoring revenue + verified supply-curve compression</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Participation 1-2%</t>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="9" ht="56" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>ADT Inc</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>5004</v>
+        <v>124308</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>6.58</v>
+        <v>151.78</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>1.38</v>
+        <v>3.63</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -7769,17 +7772,17 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Heaviest PSU%LTI in universe (90%) + verified -7.3% shrinkage</t>
+          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>Recurring monitoring revenue + verified supply-curve compression</t>
+          <t>Mega-cap recurring revenue base</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
@@ -7813,7 +7816,7 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.336</t>
+          <t>8 layers firing | cons 5.704</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
@@ -7857,7 +7860,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.812</t>
+          <t>7 layers firing | cons 5.802</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -7874,39 +7877,39 @@
     <row r="12" ht="56" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>Universal Display</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>1043</v>
+        <v>4158</v>
       </c>
       <c r="D12" s="17" t="n">
-        <v>5.29</v>
+        <v>88.94</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>0.43</v>
+        <v>2.44</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>revenue_dollar_target</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.706</t>
+          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
+          <t>OLED IP moat</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
@@ -7918,25 +7921,25 @@
     <row r="13" ht="56" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>DXC</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>DXC Technology</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>1394</v>
+        <v>1043</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>8.6</v>
+        <v>5.29</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>0.48</v>
+        <v>0.43</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -7945,61 +7948,61 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
+          <t>7 layers firing | cons 5.522</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>IT services franchise; transformation signal in PSU</t>
+          <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Participation 1-2%</t>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="14" ht="56" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>NUS</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>Nu Skin</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>1467</v>
+        <v>244</v>
       </c>
       <c r="D14" s="17" t="n">
-        <v>34.77</v>
+        <v>5.02</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>0.8</v>
+        <v>0.31</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>asset_sale_named</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.398</t>
+          <t>Named asset-sale trigger + 5-metric clean per-share stack</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
-        </is>
-      </c>
-      <c r="J14" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>P/B 0.33 + buyback shrinking organically</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
@@ -8033,7 +8036,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 5.328</t>
+          <t>7 layers firing | cons 5.332</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
@@ -8050,122 +8053,122 @@
     <row r="16" ht="56" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Universal Display</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>4158</v>
+        <v>7252</v>
       </c>
       <c r="D16" s="17" t="n">
-        <v>88.94</v>
+        <v>198.99</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>2.44</v>
+        <v>6.4</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>revenue_dollar_target</t>
+          <t>fda_phase_milestone</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
+          <t>7 layers firing | cons 5.26</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t>OLED IP moat</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>see proxy_scan + buyback_verify</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
     <row r="17" ht="56" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>NUS</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Nu Skin</t>
+          <t>DXC Technology</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
-        <v>244</v>
+        <v>1394</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>5.02</v>
+        <v>8.6</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>0.31</v>
+        <v>0.48</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>asset_sale_named</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Named asset-sale trigger + 5-metric clean per-share stack</t>
+          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>P/B 0.33 + buyback shrinking organically</t>
+          <t>IT services franchise; transformation signal in PSU</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
     <row r="18" ht="56" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>CERT</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>CERT</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>7252</v>
+        <v>862</v>
       </c>
       <c r="D18" s="17" t="n">
-        <v>198.99</v>
+        <v>5.54</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>6.4</v>
+        <v>0.84</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>fda_phase_milestone</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.87</t>
+          <t>7 layers firing | cons 5.002</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
@@ -8173,9 +8176,9 @@
           <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
-      <c r="J18" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
@@ -8209,7 +8212,7 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.85</t>
+          <t>7 layers firing | cons 4.94</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
@@ -8270,68 +8273,66 @@
     <row r="21" ht="56" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>HDSN</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Hudson Technologies</t>
+          <t>Zoetis</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>222</v>
+        <v>32997</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>5.27</v>
+        <v>78.70999999999999</v>
       </c>
       <c r="E21" s="16" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
+        <v>10.04</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
+          <t>F4 cluster + valuation + recent-incentive 60% drawdown</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>Refrigerant reclaim regulatory moat</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>Animal health franchise</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
     <row r="22" ht="56" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>HDSN</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>Hudson Technologies</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>13781</v>
+        <v>222</v>
       </c>
       <c r="D22" s="17" t="n">
-        <v>121.36</v>
+        <v>5.27</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>2.85</v>
+        <v>0.93</v>
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
@@ -8345,42 +8346,44 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.64</t>
+          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
+          <t>Refrigerant reclaim regulatory moat</t>
         </is>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>Participation 1-2%</t>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="23" ht="56" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>1074</v>
+        <v>13781</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>23.31</v>
+        <v>121.36</v>
       </c>
       <c r="E23" s="16" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="F23" s="5" t="n">
-        <v>34</v>
+        <v>2.85</v>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
@@ -8389,7 +8392,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.452</t>
+          <t>7 layers firing | cons 4.658</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
@@ -8399,41 +8402,41 @@
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
     <row r="24" ht="56" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>GIII</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>GIII</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>351</v>
+        <v>1467</v>
       </c>
       <c r="D24" s="17" t="n">
-        <v>16.44</v>
+        <v>34.77</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>ebitda_dollar_target</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>7 layers firing | cons 4.45</t>
+          <t>7 layers firing | cons 4.656</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr">
@@ -12150,10 +12153,10 @@
         <v>8</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>6.776</v>
+        <v>6.638</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -12184,10 +12187,10 @@
         <v>8</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>6.266</v>
+        <v>6.198</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
@@ -12218,7 +12221,7 @@
         <v>8</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>6.112</v>
+        <v>5.748</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-2</v>
@@ -12240,22 +12243,22 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>EPAM</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>HubSpot, Inc.</t>
+          <t>EPAM Systems, Inc.</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>5.828</v>
+        <v>6.116</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>3</v>
+        <v>-2</v>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
@@ -12264,7 +12267,7 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>PSU:4 BB:5 F4:17 RI:57</t>
+          <t>PSU:10 C10:-29 F4:18 RI:53</t>
         </is>
       </c>
     </row>
@@ -12274,22 +12277,22 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>EPAM</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>EPAM Systems, Inc.</t>
+          <t>HubSpot, Inc.</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
         <v>7</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>5.702</v>
+        <v>5.918</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -12298,7 +12301,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>PSU:10 C10:-29 F4:18 RI:53</t>
+          <t>PSU:4 BB:5 F4:17 RI:57</t>
         </is>
       </c>
     </row>
@@ -12308,31 +12311,31 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Pool Corporation</t>
+          <t>Universal Display Corporation</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>5.524</v>
+        <v>5.578</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>PSU:26 BB:5 F4:28 RI:60</t>
+          <t>PSU:39 BB:5 F4:17 RI:60</t>
         </is>
       </c>
     </row>
@@ -12342,22 +12345,22 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Universal Display Corporation</t>
+          <t>PAR Technology Corporation</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
         <v>7</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>5.432</v>
+        <v>5.176</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
@@ -12366,7 +12369,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>PSU:39 BB:5 F4:17 RI:60</t>
+          <t>PSU:16 C10:-50 RI:45 SS:35</t>
         </is>
       </c>
     </row>
@@ -12376,31 +12379,31 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>PAR Technology Corporation</t>
+          <t>Pool Corporation</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>5.25</v>
+        <v>4.88</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>PSU:16 C10:-50 RI:45 SS:35</t>
+          <t>PSU:26 BB:5 F4:28 RI:60</t>
         </is>
       </c>
     </row>
@@ -12410,31 +12413,31 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>BLND</t>
+          <t>ADT</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Blend Labs, Inc.</t>
+          <t>ADT Inc.</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
         <v>7</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>4.784</v>
+        <v>4.876</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>6</v>
+        <v>-5</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>PSU:8 BB:5 C10:-35 F4:5 RI:52 SS:20</t>
+          <t>PSU:39 BB:5 F4:12 RI:50 SS:10</t>
         </is>
       </c>
     </row>
@@ -12444,31 +12447,31 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>BLND</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>ADT Inc.</t>
+          <t>Blend Labs, Inc.</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>4.694</v>
+        <v>4.348</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>-5</v>
+        <v>5</v>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>PSU:39 BB:5 F4:12 RI:50 SS:10</t>
+          <t>PSU:8 BB:5 C10:-35 F4:5 RI:52 SS:20</t>
         </is>
       </c>
     </row>
@@ -12490,10 +12493,10 @@
         <v>7</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>4.494</v>
+        <v>4.234</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
@@ -12524,10 +12527,10 @@
         <v>6</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>5.36</v>
+        <v>5.314</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
@@ -12558,10 +12561,10 @@
         <v>6</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>4.964</v>
+        <v>5.086</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
@@ -12592,10 +12595,10 @@
         <v>6</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>4.926</v>
+        <v>4.894</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
@@ -12614,31 +12617,31 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>NUS</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Nu Skin Enterprises, Inc.</t>
+          <t>DXC Technology Company</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>4.834</v>
+        <v>4.876</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-2</v>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Consumer Defensive</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>PSU:48 BB:5 C10:-32 RI:53</t>
+          <t>PSU:40 BB:5 RI:57</t>
         </is>
       </c>
     </row>
@@ -12648,31 +12651,31 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>SharpLink, Inc.</t>
+          <t>Zoetis Inc.</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>4.79</v>
+        <v>4.732</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>-8</v>
+        <v>1</v>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>PSU:22 C10:15 RI:71</t>
+          <t>PSU:8 BB:5 C10:-3 F4:12 RI:60</t>
         </is>
       </c>
     </row>
@@ -12682,31 +12685,31 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>DXC</t>
+          <t>IQV</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>DXC Technology Company</t>
+          <t>IQVIA Holdings, Inc.</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E21" s="16" t="n">
-        <v>4.724</v>
+        <v>4.726</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>-8</v>
+        <v>22</v>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>PSU:40 BB:5 RI:57</t>
+          <t>PSU:4 BB:5 C10:43 RI:51 SS:21</t>
         </is>
       </c>
     </row>
@@ -12716,22 +12719,22 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>MSCI Inc.</t>
+          <t>SharpLink, Inc.</t>
         </is>
       </c>
       <c r="D22" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>4.542</v>
+        <v>4.688</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>21</v>
+        <v>-9</v>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
@@ -12740,7 +12743,7 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>PSU:35 BB:8 C10:-26 F4:16 RI:16</t>
+          <t>PSU:22 C10:15 RI:71</t>
         </is>
       </c>
     </row>
@@ -12762,10 +12765,10 @@
         <v>6</v>
       </c>
       <c r="E23" s="16" t="n">
-        <v>4.482</v>
+        <v>4.61</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
@@ -12784,31 +12787,31 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>IQV</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>IQVIA Holdings, Inc.</t>
+          <t>MSCI Inc.</t>
         </is>
       </c>
       <c r="D24" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>4.4</v>
+        <v>4.478</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>PSU:4 BB:5 C10:43 RI:51 SS:21</t>
+          <t>PSU:35 BB:8 C10:-26 F4:16 RI:16</t>
         </is>
       </c>
     </row>
@@ -12818,31 +12821,31 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>KMX</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Mastercard Incorporated</t>
+          <t>CarMax Inc</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E25" s="16" t="n">
-        <v>4.364</v>
+        <v>4.458</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>PSU:32 BB:5 C10:78 RI:50</t>
+          <t>PSU:30 BB:8 RI:33</t>
         </is>
       </c>
     </row>
@@ -12852,31 +12855,31 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>KMPR</t>
+          <t>OPCH</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Kemper Corporation</t>
+          <t>Option Care Health, Inc.</t>
         </is>
       </c>
       <c r="D26" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E26" s="17" t="n">
-        <v>4.336</v>
+        <v>4.448</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>-6</v>
+        <v>26</v>
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>PSU:27 BB:8 C10:20 RI:65</t>
+          <t>PSU:24 BB:5 C10:-1 F4:23 RI:52</t>
         </is>
       </c>
     </row>
@@ -12886,22 +12889,22 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>KMX</t>
+          <t>APTV</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>CarMax Inc</t>
+          <t>Aptiv PLC</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E27" s="16" t="n">
-        <v>4.3</v>
+        <v>4.43</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
@@ -12910,7 +12913,7 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>PSU:30 BB:8 RI:33</t>
+          <t>PSU:40 BB:5 RI:35</t>
         </is>
       </c>
     </row>
@@ -12920,31 +12923,31 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>APTV</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Aptiv PLC</t>
+          <t>Mastercard Incorporated</t>
         </is>
       </c>
       <c r="D28" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="17" t="n">
-        <v>4.268</v>
+        <v>4.314</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>PSU:40 BB:5 RI:35</t>
+          <t>PSU:32 BB:5 C10:78 RI:50</t>
         </is>
       </c>
     </row>
@@ -12954,31 +12957,31 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>NUS</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Zoetis Inc.</t>
+          <t>Nu Skin Enterprises, Inc.</t>
         </is>
       </c>
       <c r="D29" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E29" s="16" t="n">
-        <v>4.254</v>
+        <v>4.296</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>-3</v>
+        <v>-15</v>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Consumer Defensive</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>PSU:8 BB:5 C10:-3 F4:12 RI:60</t>
+          <t>PSU:48 BB:5 C10:-32 RI:53</t>
         </is>
       </c>
     </row>
@@ -13000,7 +13003,7 @@
         <v>6</v>
       </c>
       <c r="E30" s="17" t="n">
-        <v>4.032</v>
+        <v>4.224</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>-15</v>
@@ -13022,31 +13025,31 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>ACM</t>
+          <t>KMPR</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>Kemper Corporation</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="16" t="n">
-        <v>3.996</v>
+        <v>4.144</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>17</v>
+        <v>-11</v>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>BB:5 F4:6 RI:54</t>
+          <t>PSU:27 BB:8 C10:20 RI:65</t>
         </is>
       </c>
     </row>
@@ -13056,22 +13059,22 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>AZTA</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Option Care Health, Inc.</t>
+          <t>Azenta, Inc.</t>
         </is>
       </c>
       <c r="D32" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E32" s="17" t="n">
-        <v>3.954</v>
+        <v>4.126</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>9</v>
+        <v>-6</v>
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
@@ -13080,7 +13083,7 @@
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t>PSU:24 BB:5 C10:-1 F4:23 RI:52</t>
+          <t>PSU:29</t>
         </is>
       </c>
     </row>
@@ -13090,31 +13093,31 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>NSP</t>
+          <t>MGPI</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Insperity, Inc.</t>
+          <t>MGP Ingredients, Inc.</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="16" t="n">
-        <v>3.934</v>
+        <v>4.012</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>25</v>
+        <v>-8</v>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Defensive</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>PSU:43 F4:28 RI:40</t>
+          <t>PSU:30 RI:46</t>
         </is>
       </c>
     </row>
@@ -13124,31 +13127,31 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>TSEOF</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Azenta, Inc.</t>
+          <t>Trinseo PLC</t>
         </is>
       </c>
       <c r="D34" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="17" t="n">
-        <v>3.918</v>
-      </c>
-      <c r="F34" s="8" t="n">
-        <v>-11</v>
+        <v>4.01</v>
+      </c>
+      <c r="F34" s="19" t="n">
+        <v>66</v>
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t>PSU:29</t>
+          <t>PSU:17 C10:-10 RI:40 SS:55</t>
         </is>
       </c>
     </row>
@@ -13282,7 +13285,7 @@
           <t>Repay Holdings Corporation</t>
         </is>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="20" t="n">
         <v>68</v>
       </c>
       <c r="E5" s="5" t="n">
@@ -13296,7 +13299,7 @@
       <c r="G5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="20" t="n">
+      <c r="H5" s="21" t="n">
         <v>44</v>
       </c>
       <c r="I5" s="16" t="n">
@@ -13322,7 +13325,7 @@
           <t>Gossamer Bio, Inc.</t>
         </is>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="20" t="n">
         <v>61</v>
       </c>
       <c r="E6" s="8" t="n">
@@ -13336,7 +13339,7 @@
       <c r="G6" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="21" t="n">
+      <c r="H6" s="22" t="n">
         <v>96</v>
       </c>
       <c r="I6" s="17" t="n">
@@ -13362,7 +13365,7 @@
           <t>ZoomInfo Technologies Inc.</t>
         </is>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="20" t="n">
         <v>60</v>
       </c>
       <c r="E7" s="5" t="n">
@@ -13376,7 +13379,7 @@
       <c r="G7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="20" t="n">
+      <c r="H7" s="21" t="n">
         <v>78</v>
       </c>
       <c r="I7" s="16" t="n">
@@ -13402,7 +13405,7 @@
           <t>Goosehead Insurance, Inc.</t>
         </is>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="20" t="n">
         <v>53</v>
       </c>
       <c r="E8" s="8" t="n">
@@ -13416,7 +13419,7 @@
       <c r="G8" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="21" t="n">
+      <c r="H8" s="22" t="n">
         <v>70</v>
       </c>
       <c r="I8" s="17" t="n">
@@ -13442,7 +13445,7 @@
           <t>Guidewire Software, Inc.</t>
         </is>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="20" t="n">
         <v>53</v>
       </c>
       <c r="E9" s="5" t="n">
@@ -13456,7 +13459,7 @@
       <c r="G9" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="20" t="n">
+      <c r="H9" s="21" t="n">
         <v>60</v>
       </c>
       <c r="I9" s="16" t="n">
@@ -13482,7 +13485,7 @@
           <t>Comtech Telecommunications Corp</t>
         </is>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="20" t="n">
         <v>52</v>
       </c>
       <c r="E10" s="8" t="n">
@@ -13496,7 +13499,7 @@
       <c r="G10" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="21" t="n">
+      <c r="H10" s="22" t="n">
         <v>61</v>
       </c>
       <c r="I10" s="17" t="n">
@@ -13522,7 +13525,7 @@
           <t>BiomX Inc.</t>
         </is>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="20" t="n">
         <v>52</v>
       </c>
       <c r="E11" s="5" t="n">
@@ -13536,7 +13539,7 @@
       <c r="G11" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="20" t="n">
+      <c r="H11" s="21" t="n">
         <v>96</v>
       </c>
       <c r="I11" s="16" t="n">
@@ -13562,7 +13565,7 @@
           <t>ChargePoint Holdings, Inc.</t>
         </is>
       </c>
-      <c r="D12" s="19" t="n">
+      <c r="D12" s="20" t="n">
         <v>52</v>
       </c>
       <c r="E12" s="8" t="n">
@@ -13576,7 +13579,7 @@
       <c r="G12" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="21" t="n">
+      <c r="H12" s="22" t="n">
         <v>49</v>
       </c>
       <c r="I12" s="17" t="n">
@@ -13602,7 +13605,7 @@
           <t>DXC Technology Company</t>
         </is>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="20" t="n">
         <v>52</v>
       </c>
       <c r="E13" s="5" t="n">
@@ -13616,7 +13619,7 @@
       <c r="G13" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="20" t="n">
+      <c r="H13" s="21" t="n">
         <v>48</v>
       </c>
       <c r="I13" s="16" t="n">
@@ -13642,7 +13645,7 @@
           <t>Processa Pharmaceuticals, Inc.</t>
         </is>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="20" t="n">
         <v>51</v>
       </c>
       <c r="E14" s="8" t="n">
@@ -13656,7 +13659,7 @@
       <c r="G14" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="H14" s="21" t="n">
+      <c r="H14" s="22" t="n">
         <v>86</v>
       </c>
       <c r="I14" s="17" t="n">
@@ -13682,7 +13685,7 @@
           <t>Peabody Energy Corporation</t>
         </is>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="20" t="n">
         <v>51</v>
       </c>
       <c r="E15" s="5" t="n">
@@ -13696,7 +13699,7 @@
       <c r="G15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="20" t="n">
+      <c r="H15" s="21" t="n">
         <v>36</v>
       </c>
       <c r="I15" s="16" t="n">
@@ -13722,7 +13725,7 @@
           <t>Ready Capital Corporation</t>
         </is>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="20" t="n">
         <v>49</v>
       </c>
       <c r="E16" s="8" t="n">
@@ -13736,7 +13739,7 @@
       <c r="G16" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="21" t="n">
+      <c r="H16" s="22" t="n">
         <v>63</v>
       </c>
       <c r="I16" s="17" t="n">
@@ -13762,7 +13765,7 @@
           <t>Kingsway Corporation</t>
         </is>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="20" t="n">
         <v>49</v>
       </c>
       <c r="E17" s="5" t="n">
@@ -13776,7 +13779,7 @@
       <c r="G17" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H17" s="20" t="n">
+      <c r="H17" s="21" t="n">
         <v>39</v>
       </c>
       <c r="I17" s="16" t="n">
@@ -13802,7 +13805,7 @@
           <t>Heron Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="D18" s="19" t="n">
+      <c r="D18" s="20" t="n">
         <v>48</v>
       </c>
       <c r="E18" s="8" t="n">
@@ -13816,7 +13819,7 @@
       <c r="G18" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="21" t="n">
+      <c r="H18" s="22" t="n">
         <v>82</v>
       </c>
       <c r="I18" s="17" t="n">
@@ -13842,7 +13845,7 @@
           <t>Standard BioTools Inc.</t>
         </is>
       </c>
-      <c r="D19" s="19" t="n">
+      <c r="D19" s="20" t="n">
         <v>48</v>
       </c>
       <c r="E19" s="5" t="n">
@@ -13856,7 +13859,7 @@
       <c r="G19" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H19" s="20" t="n">
+      <c r="H19" s="21" t="n">
         <v>52</v>
       </c>
       <c r="I19" s="16" t="n">
@@ -13882,7 +13885,7 @@
           <t>InspireMD Inc.</t>
         </is>
       </c>
-      <c r="D20" s="19" t="n">
+      <c r="D20" s="20" t="n">
         <v>47</v>
       </c>
       <c r="E20" s="8" t="n">
@@ -13896,7 +13899,7 @@
       <c r="G20" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="21" t="n">
+      <c r="H20" s="22" t="n">
         <v>76</v>
       </c>
       <c r="I20" s="17" t="n">
@@ -13922,7 +13925,7 @@
           <t>Rein Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="D21" s="19" t="n">
+      <c r="D21" s="20" t="n">
         <v>46</v>
       </c>
       <c r="E21" s="5" t="n">
@@ -13936,7 +13939,7 @@
       <c r="G21" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="20" t="n">
+      <c r="H21" s="21" t="n">
         <v>58</v>
       </c>
       <c r="I21" s="16" t="n">
@@ -13962,7 +13965,7 @@
           <t>Booz Allen Hamilton Holding Cor</t>
         </is>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D22" s="20" t="n">
         <v>46</v>
       </c>
       <c r="E22" s="8" t="n">
@@ -13976,7 +13979,7 @@
       <c r="G22" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="21" t="n">
+      <c r="H22" s="22" t="n">
         <v>45</v>
       </c>
       <c r="I22" s="17" t="n">
@@ -14002,7 +14005,7 @@
           <t>VolitionRX Limited</t>
         </is>
       </c>
-      <c r="D23" s="19" t="n">
+      <c r="D23" s="20" t="n">
         <v>45</v>
       </c>
       <c r="E23" s="5" t="n">
@@ -14016,7 +14019,7 @@
       <c r="G23" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="20" t="n">
+      <c r="H23" s="21" t="n">
         <v>92</v>
       </c>
       <c r="I23" s="16" t="n">
@@ -14042,7 +14045,7 @@
           <t>Total Return Securities Fund</t>
         </is>
       </c>
-      <c r="D24" s="19" t="n">
+      <c r="D24" s="20" t="n">
         <v>44</v>
       </c>
       <c r="E24" s="8" t="n">
@@ -14056,7 +14059,7 @@
       <c r="G24" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H24" s="21" t="n">
+      <c r="H24" s="22" t="n">
         <v>8</v>
       </c>
       <c r="I24" s="17" t="n">
@@ -14082,7 +14085,7 @@
           <t>Fox Corporation</t>
         </is>
       </c>
-      <c r="D25" s="19" t="n">
+      <c r="D25" s="20" t="n">
         <v>44</v>
       </c>
       <c r="E25" s="5" t="n">
@@ -14096,7 +14099,7 @@
       <c r="G25" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H25" s="20" t="n">
+      <c r="H25" s="21" t="n">
         <v>31</v>
       </c>
       <c r="I25" s="16" t="n">
@@ -14122,7 +14125,7 @@
           <t>Outlook Therapeutics, Inc.</t>
         </is>
       </c>
-      <c r="D26" s="19" t="n">
+      <c r="D26" s="20" t="n">
         <v>44</v>
       </c>
       <c r="E26" s="8" t="n">
@@ -14136,7 +14139,7 @@
       <c r="G26" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="H26" s="21" t="n">
+      <c r="H26" s="22" t="n">
         <v>53</v>
       </c>
       <c r="I26" s="17" t="n">
@@ -14162,7 +14165,7 @@
           <t>My Size, Inc.</t>
         </is>
       </c>
-      <c r="D27" s="19" t="n">
+      <c r="D27" s="20" t="n">
         <v>43</v>
       </c>
       <c r="E27" s="5" t="n">
@@ -14176,7 +14179,7 @@
       <c r="G27" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="20" t="n">
+      <c r="H27" s="21" t="n">
         <v>72</v>
       </c>
       <c r="I27" s="16" t="n">
@@ -14202,7 +14205,7 @@
           <t>Purple Innovation, Inc.</t>
         </is>
       </c>
-      <c r="D28" s="19" t="n">
+      <c r="D28" s="20" t="n">
         <v>43</v>
       </c>
       <c r="E28" s="8" t="n">
@@ -14216,7 +14219,7 @@
       <c r="G28" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="21" t="n">
+      <c r="H28" s="22" t="n">
         <v>66</v>
       </c>
       <c r="I28" s="17" t="n">
@@ -14242,7 +14245,7 @@
           <t>Cosmos Health Inc.</t>
         </is>
       </c>
-      <c r="D29" s="19" t="n">
+      <c r="D29" s="20" t="n">
         <v>43</v>
       </c>
       <c r="E29" s="5" t="n">
@@ -14256,7 +14259,7 @@
       <c r="G29" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H29" s="20" t="n">
+      <c r="H29" s="21" t="n">
         <v>84</v>
       </c>
       <c r="I29" s="16" t="n">
@@ -14282,7 +14285,7 @@
           <t>Power Solutions International,</t>
         </is>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D30" s="20" t="n">
         <v>43</v>
       </c>
       <c r="E30" s="8" t="n">
@@ -14296,7 +14299,7 @@
       <c r="G30" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H30" s="21" t="n">
+      <c r="H30" s="22" t="n">
         <v>67</v>
       </c>
       <c r="I30" s="17" t="n">
@@ -14322,7 +14325,7 @@
           <t>NexGel, Inc</t>
         </is>
       </c>
-      <c r="D31" s="19" t="n">
+      <c r="D31" s="20" t="n">
         <v>43</v>
       </c>
       <c r="E31" s="5" t="n">
@@ -14336,7 +14339,7 @@
       <c r="G31" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H31" s="20" t="n">
+      <c r="H31" s="21" t="n">
         <v>80</v>
       </c>
       <c r="I31" s="16" t="n">
@@ -14362,7 +14365,7 @@
           <t>Salesforce, Inc.</t>
         </is>
       </c>
-      <c r="D32" s="19" t="n">
+      <c r="D32" s="20" t="n">
         <v>42</v>
       </c>
       <c r="E32" s="8" t="n">
@@ -14376,7 +14379,7 @@
       <c r="G32" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H32" s="21" t="n">
+      <c r="H32" s="22" t="n">
         <v>45</v>
       </c>
       <c r="I32" s="17" t="n">
@@ -14402,7 +14405,7 @@
           <t>Vitesse Energy, Inc.</t>
         </is>
       </c>
-      <c r="D33" s="19" t="n">
+      <c r="D33" s="20" t="n">
         <v>42</v>
       </c>
       <c r="E33" s="5" t="n">
@@ -14416,7 +14419,7 @@
       <c r="G33" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H33" s="20" t="n">
+      <c r="H33" s="21" t="n">
         <v>41</v>
       </c>
       <c r="I33" s="16" t="n">
@@ -14442,7 +14445,7 @@
           <t>Krispy Kreme, Inc.</t>
         </is>
       </c>
-      <c r="D34" s="19" t="n">
+      <c r="D34" s="20" t="n">
         <v>42</v>
       </c>
       <c r="E34" s="8" t="n">
@@ -14456,7 +14459,7 @@
       <c r="G34" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H34" s="21" t="n">
+      <c r="H34" s="22" t="n">
         <v>37</v>
       </c>
       <c r="I34" s="17" t="n">
@@ -14482,7 +14485,7 @@
           <t>Nerdy Inc.</t>
         </is>
       </c>
-      <c r="D35" s="19" t="n">
+      <c r="D35" s="20" t="n">
         <v>41</v>
       </c>
       <c r="E35" s="5" t="n">
@@ -14496,7 +14499,7 @@
       <c r="G35" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H35" s="20" t="n">
+      <c r="H35" s="21" t="n">
         <v>51</v>
       </c>
       <c r="I35" s="16" t="n">
@@ -14522,7 +14525,7 @@
           <t>Artiva Biotherapeutics, Inc.</t>
         </is>
       </c>
-      <c r="D36" s="19" t="n">
+      <c r="D36" s="20" t="n">
         <v>41</v>
       </c>
       <c r="E36" s="8" t="n">
@@ -14536,7 +14539,7 @@
       <c r="G36" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H36" s="21" t="n">
+      <c r="H36" s="22" t="n">
         <v>49</v>
       </c>
       <c r="I36" s="17" t="n">
@@ -14562,7 +14565,7 @@
           <t>STERIS plc (Ireland)</t>
         </is>
       </c>
-      <c r="D37" s="19" t="n">
+      <c r="D37" s="20" t="n">
         <v>41</v>
       </c>
       <c r="E37" s="5" t="n">
@@ -14576,7 +14579,7 @@
       <c r="G37" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H37" s="20" t="n">
+      <c r="H37" s="21" t="n">
         <v>25</v>
       </c>
       <c r="I37" s="16" t="n">
@@ -14602,7 +14605,7 @@
           <t>Rubrik, Inc.</t>
         </is>
       </c>
-      <c r="D38" s="19" t="n">
+      <c r="D38" s="20" t="n">
         <v>41</v>
       </c>
       <c r="E38" s="8" t="n">
@@ -14616,7 +14619,7 @@
       <c r="G38" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H38" s="21" t="n">
+      <c r="H38" s="22" t="n">
         <v>30</v>
       </c>
       <c r="I38" s="17" t="n">
@@ -14642,7 +14645,7 @@
           <t>Medline Inc.</t>
         </is>
       </c>
-      <c r="D39" s="19" t="n">
+      <c r="D39" s="20" t="n">
         <v>40</v>
       </c>
       <c r="E39" s="5" t="n">
@@ -14656,7 +14659,7 @@
       <c r="G39" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H39" s="20" t="n">
+      <c r="H39" s="21" t="n">
         <v>29</v>
       </c>
       <c r="I39" s="16" t="n">
@@ -14682,7 +14685,7 @@
           <t>Toro Corp.</t>
         </is>
       </c>
-      <c r="D40" s="19" t="n">
+      <c r="D40" s="20" t="n">
         <v>40</v>
       </c>
       <c r="E40" s="8" t="n">
@@ -14696,7 +14699,7 @@
       <c r="G40" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H40" s="21" t="n">
+      <c r="H40" s="22" t="n">
         <v>40</v>
       </c>
       <c r="I40" s="17" t="n">
@@ -14722,7 +14725,7 @@
           <t>CuriosityStream Inc.</t>
         </is>
       </c>
-      <c r="D41" s="19" t="n">
+      <c r="D41" s="20" t="n">
         <v>40</v>
       </c>
       <c r="E41" s="5" t="n">
@@ -14736,7 +14739,7 @@
       <c r="G41" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H41" s="20" t="n">
+      <c r="H41" s="21" t="n">
         <v>57</v>
       </c>
       <c r="I41" s="16" t="n">
@@ -14762,7 +14765,7 @@
           <t>Health Catalyst, Inc</t>
         </is>
       </c>
-      <c r="D42" s="19" t="n">
+      <c r="D42" s="20" t="n">
         <v>40</v>
       </c>
       <c r="E42" s="8" t="n">
@@ -14776,7 +14779,7 @@
       <c r="G42" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H42" s="21" t="n">
+      <c r="H42" s="22" t="n">
         <v>55</v>
       </c>
       <c r="I42" s="17" t="n">
@@ -14816,7 +14819,7 @@
       <c r="G43" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H43" s="20" t="n">
+      <c r="H43" s="21" t="n">
         <v>87</v>
       </c>
       <c r="I43" s="16" t="n">
@@ -14856,7 +14859,7 @@
       <c r="G44" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H44" s="21" t="n">
+      <c r="H44" s="22" t="n">
         <v>63</v>
       </c>
       <c r="I44" s="17" t="n">
@@ -14995,7 +14998,7 @@
       <c r="F5" s="16" t="n">
         <v>5.854111</v>
       </c>
-      <c r="G5" s="20" t="n">
+      <c r="G5" s="21" t="n">
         <v>11.4700004</v>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -15031,7 +15034,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="22" t="n">
         <v>-12.622</v>
       </c>
       <c r="H6" s="10" t="inlineStr">
@@ -15065,7 +15068,7 @@
       <c r="F7" s="16" t="n">
         <v>6.5333333</v>
       </c>
-      <c r="G7" s="20" t="n">
+      <c r="G7" s="21" t="n">
         <v>4.2069998</v>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -15099,7 +15102,7 @@
       <c r="F8" s="17" t="n">
         <v>4.679035</v>
       </c>
-      <c r="G8" s="21" t="n">
+      <c r="G8" s="22" t="n">
         <v>19.077998</v>
       </c>
       <c r="H8" s="10" t="inlineStr">
@@ -15135,7 +15138,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G9" s="20" t="n">
+      <c r="G9" s="21" t="n">
         <v>0.10899999</v>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -15169,7 +15172,7 @@
       <c r="F10" s="17" t="n">
         <v>17.51089</v>
       </c>
-      <c r="G10" s="21" t="n">
+      <c r="G10" s="22" t="n">
         <v>6.4109996</v>
       </c>
       <c r="H10" s="10" t="inlineStr">
@@ -15203,7 +15206,7 @@
       <c r="F11" s="16" t="n">
         <v>9.148345000000001</v>
       </c>
-      <c r="G11" s="20" t="n">
+      <c r="G11" s="21" t="n">
         <v>10.233</v>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -15239,7 +15242,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G12" s="21" t="n">
+      <c r="G12" s="22" t="n">
         <v>-2.8499998</v>
       </c>
       <c r="H12" s="10" t="inlineStr">
@@ -15273,7 +15276,7 @@
       <c r="F13" s="16" t="n">
         <v>19.150717</v>
       </c>
-      <c r="G13" s="20" t="n">
+      <c r="G13" s="21" t="n">
         <v>3.3069998</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -15309,7 +15312,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G14" s="21" t="n">
+      <c r="G14" s="22" t="n">
         <v>-9.856</v>
       </c>
       <c r="H14" s="10" t="inlineStr">
@@ -15343,7 +15346,7 @@
       <c r="F15" s="16" t="n">
         <v>9.943130500000001</v>
       </c>
-      <c r="G15" s="20" t="n">
+      <c r="G15" s="21" t="n">
         <v>8.282</v>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -15377,7 +15380,7 @@
       <c r="F16" s="17" t="n">
         <v>12.411422</v>
       </c>
-      <c r="G16" s="21" t="n">
+      <c r="G16" s="22" t="n">
         <v>8.5</v>
       </c>
       <c r="H16" s="10" t="inlineStr">
@@ -15411,7 +15414,7 @@
       <c r="F17" s="16" t="n">
         <v>166.7683</v>
       </c>
-      <c r="G17" s="20" t="n">
+      <c r="G17" s="21" t="n">
         <v>0.75</v>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -15445,7 +15448,7 @@
       <c r="F18" s="17" t="n">
         <v>14.648475</v>
       </c>
-      <c r="G18" s="21" t="n">
+      <c r="G18" s="22" t="n">
         <v>2.8110001</v>
       </c>
       <c r="H18" s="10" t="inlineStr">
@@ -15479,7 +15482,7 @@
       <c r="F19" s="16" t="n">
         <v>10.444035</v>
       </c>
-      <c r="G19" s="20" t="n">
+      <c r="G19" s="21" t="n">
         <v>7.056</v>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -15513,7 +15516,7 @@
       <c r="F20" s="17" t="n">
         <v>8.47991</v>
       </c>
-      <c r="G20" s="21" t="n">
+      <c r="G20" s="22" t="n">
         <v>7.566000000000001</v>
       </c>
       <c r="H20" s="10" t="inlineStr">
@@ -15547,7 +15550,7 @@
       <c r="F21" s="16" t="n">
         <v>7.682529</v>
       </c>
-      <c r="G21" s="20" t="n">
+      <c r="G21" s="21" t="n">
         <v>12.528</v>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -15581,7 +15584,7 @@
       <c r="F22" s="17" t="n">
         <v>8.268003999999999</v>
       </c>
-      <c r="G22" s="21" t="n">
+      <c r="G22" s="22" t="n">
         <v>12.644</v>
       </c>
       <c r="H22" s="10" t="inlineStr">
@@ -15615,7 +15618,7 @@
       <c r="F23" s="16" t="n">
         <v>9.176824</v>
       </c>
-      <c r="G23" s="20" t="n">
+      <c r="G23" s="21" t="n">
         <v>12.286</v>
       </c>
       <c r="H23" s="7" t="inlineStr">
@@ -15649,7 +15652,7 @@
       <c r="F24" s="17" t="n">
         <v>9.315649000000001</v>
       </c>
-      <c r="G24" s="21" t="n">
+      <c r="G24" s="22" t="n">
         <v>12.94</v>
       </c>
       <c r="H24" s="10" t="inlineStr">
@@ -15683,7 +15686,7 @@
       <c r="F25" s="16" t="n">
         <v>6.766146</v>
       </c>
-      <c r="G25" s="20" t="n">
+      <c r="G25" s="21" t="n">
         <v>11.607</v>
       </c>
       <c r="H25" s="7" t="inlineStr">
@@ -15721,7 +15724,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G26" s="21" t="n">
+      <c r="G26" s="22" t="n">
         <v>61.172</v>
       </c>
       <c r="H26" s="10" t="inlineStr">
@@ -15759,7 +15762,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G27" s="20" t="n">
+      <c r="G27" s="21" t="n">
         <v>7.478999999999999</v>
       </c>
       <c r="H27" s="7" t="inlineStr">
@@ -15797,7 +15800,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G28" s="21" t="n">
+      <c r="G28" s="22" t="n">
         <v>4.777</v>
       </c>
       <c r="H28" s="10" t="inlineStr">
@@ -15835,7 +15838,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G29" s="20" t="n">
+      <c r="G29" s="21" t="n">
         <v>-5.933999999999999</v>
       </c>
       <c r="H29" s="7" t="inlineStr">
@@ -15873,7 +15876,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G30" s="21" t="n">
+      <c r="G30" s="22" t="n">
         <v>-2.5710002</v>
       </c>
       <c r="H30" s="10" t="inlineStr">
@@ -15911,7 +15914,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G31" s="20" t="n">
+      <c r="G31" s="21" t="n">
         <v>5.252</v>
       </c>
       <c r="H31" s="7" t="inlineStr">
@@ -15949,7 +15952,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G32" s="21" t="n">
+      <c r="G32" s="22" t="n">
         <v>7.2129995</v>
       </c>
       <c r="H32" s="10" t="inlineStr">
@@ -15987,7 +15990,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G33" s="20" t="n">
+      <c r="G33" s="21" t="n">
         <v>2.609</v>
       </c>
       <c r="H33" s="7" t="inlineStr">
@@ -16025,7 +16028,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G34" s="21" t="n">
+      <c r="G34" s="22" t="n">
         <v>13.207</v>
       </c>
       <c r="H34" s="10" t="inlineStr">
@@ -16063,7 +16066,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G35" s="20" t="n">
+      <c r="G35" s="21" t="n">
         <v>16.758</v>
       </c>
       <c r="H35" s="7" t="inlineStr">
@@ -16097,7 +16100,7 @@
       <c r="F36" s="17" t="n">
         <v>7.927419</v>
       </c>
-      <c r="G36" s="21" t="n">
+      <c r="G36" s="22" t="n">
         <v>0</v>
       </c>
       <c r="H36" s="10" t="inlineStr">
@@ -16131,7 +16134,7 @@
       <c r="F37" s="16" t="n">
         <v>11.657143</v>
       </c>
-      <c r="G37" s="20" t="n">
+      <c r="G37" s="21" t="n">
         <v>7.823</v>
       </c>
       <c r="H37" s="7" t="inlineStr">
@@ -16165,7 +16168,7 @@
       <c r="F38" s="17" t="n">
         <v>20.921429</v>
       </c>
-      <c r="G38" s="21" t="n">
+      <c r="G38" s="22" t="n">
         <v>3.918999799999999</v>
       </c>
       <c r="H38" s="10" t="inlineStr">
@@ -16199,7 +16202,7 @@
       <c r="F39" s="16" t="n">
         <v>11.634099</v>
       </c>
-      <c r="G39" s="20" t="n">
+      <c r="G39" s="21" t="n">
         <v>7.754</v>
       </c>
       <c r="H39" s="7" t="inlineStr">
@@ -16237,7 +16240,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G40" s="21" t="n">
+      <c r="G40" s="22" t="n">
         <v>18.855</v>
       </c>
       <c r="H40" s="10" t="inlineStr">
@@ -16275,7 +16278,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G41" s="20" t="n">
+      <c r="G41" s="21" t="n">
         <v>7.539999999999999</v>
       </c>
       <c r="H41" s="7" t="inlineStr">
@@ -16313,7 +16316,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G42" s="21" t="n">
+      <c r="G42" s="22" t="n">
         <v>1.125</v>
       </c>
       <c r="H42" s="10" t="inlineStr">
@@ -16351,7 +16354,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G43" s="20" t="n">
+      <c r="G43" s="21" t="n">
         <v>9.097</v>
       </c>
       <c r="H43" s="7" t="inlineStr">
@@ -16389,7 +16392,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G44" s="21" t="n">
+      <c r="G44" s="22" t="n">
         <v>8.518000000000001</v>
       </c>
       <c r="H44" s="10" t="inlineStr">
@@ -16427,7 +16430,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G45" s="20" t="n">
+      <c r="G45" s="21" t="n">
         <v>9.991</v>
       </c>
       <c r="H45" s="7" t="inlineStr">
@@ -16465,7 +16468,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G46" s="21" t="n">
+      <c r="G46" s="22" t="n">
         <v>18.855</v>
       </c>
       <c r="H46" s="10" t="inlineStr">
@@ -16503,7 +16506,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G47" s="20" t="n">
+      <c r="G47" s="21" t="n">
         <v>3.85</v>
       </c>
       <c r="H47" s="7" t="inlineStr">
@@ -16541,7 +16544,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G48" s="21" t="n">
+      <c r="G48" s="22" t="n">
         <v>7.2270006</v>
       </c>
       <c r="H48" s="10" t="inlineStr">
@@ -16579,7 +16582,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G49" s="20" t="n">
+      <c r="G49" s="21" t="n">
         <v>18.671</v>
       </c>
       <c r="H49" s="7" t="inlineStr">
@@ -16617,7 +16620,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G50" s="21" t="n">
+      <c r="G50" s="22" t="n">
         <v>14.094</v>
       </c>
       <c r="H50" s="10" t="inlineStr">
@@ -16655,7 +16658,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G51" s="20" t="n">
+      <c r="G51" s="21" t="n">
         <v>6.414000000000001</v>
       </c>
       <c r="H51" s="7" t="inlineStr">
@@ -16693,7 +16696,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G52" s="21" t="n">
+      <c r="G52" s="22" t="n">
         <v>10.064</v>
       </c>
       <c r="H52" s="10" t="inlineStr">
@@ -16731,7 +16734,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G53" s="20" t="n">
+      <c r="G53" s="21" t="n">
         <v>7.435</v>
       </c>
       <c r="H53" s="7" t="inlineStr">
@@ -16769,7 +16772,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G54" s="21" t="n">
+      <c r="G54" s="22" t="n">
         <v>21.757999</v>
       </c>
       <c r="H54" s="10" t="inlineStr">
@@ -16807,7 +16810,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G55" s="20" t="n">
+      <c r="G55" s="21" t="n">
         <v>10.922</v>
       </c>
       <c r="H55" s="7" t="inlineStr">
@@ -16845,7 +16848,7 @@
           <t>–</t>
         </is>
       </c>
-      <c r="G56" s="21" t="n">
+      <c r="G56" s="22" t="n">
         <v>21.345</v>
       </c>
       <c r="H56" s="10" t="inlineStr">
@@ -16879,7 +16882,7 @@
       <c r="F57" s="16" t="n">
         <v>12.022634</v>
       </c>
-      <c r="G57" s="20" t="n">
+      <c r="G57" s="21" t="n">
         <v>10.697</v>
       </c>
       <c r="H57" s="7" t="inlineStr">
@@ -16913,7 +16916,7 @@
       <c r="F58" s="17" t="n">
         <v>29.628126</v>
       </c>
-      <c r="G58" s="21" t="n">
+      <c r="G58" s="22" t="n">
         <v>5.842</v>
       </c>
       <c r="H58" s="10" t="inlineStr">
@@ -16947,7 +16950,7 @@
       <c r="F59" s="16" t="n">
         <v>20.560537</v>
       </c>
-      <c r="G59" s="20" t="n">
+      <c r="G59" s="21" t="n">
         <v>30.955</v>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -16981,7 +16984,7 @@
       <c r="F60" s="17" t="n">
         <v>15.749999</v>
       </c>
-      <c r="G60" s="21" t="n">
+      <c r="G60" s="22" t="n">
         <v>11.611</v>
       </c>
       <c r="H60" s="10" t="inlineStr">
@@ -17015,7 +17018,7 @@
       <c r="F61" s="16" t="n">
         <v>27.900793</v>
       </c>
-      <c r="G61" s="20" t="n">
+      <c r="G61" s="21" t="n">
         <v>23.482999</v>
       </c>
       <c r="H61" s="7" t="inlineStr">
@@ -17049,7 +17052,7 @@
       <c r="F62" s="17" t="n">
         <v>13.897888</v>
       </c>
-      <c r="G62" s="21" t="n">
+      <c r="G62" s="22" t="n">
         <v>40.905997</v>
       </c>
       <c r="H62" s="10" t="inlineStr">
@@ -17083,7 +17086,7 @@
       <c r="F63" s="16" t="n">
         <v>13.429799</v>
       </c>
-      <c r="G63" s="20" t="n">
+      <c r="G63" s="21" t="n">
         <v>15.824</v>
       </c>
       <c r="H63" s="7" t="inlineStr">
@@ -17117,7 +17120,7 @@
       <c r="F64" s="17" t="n">
         <v>12.046511</v>
       </c>
-      <c r="G64" s="21" t="n">
+      <c r="G64" s="22" t="n">
         <v>9.552</v>
       </c>
       <c r="H64" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Workbook copy: dynamic layer count + updated layer roster
The Contents/Methodology/Correlation copy hardcoded "30 layers" while
the consensus has grown to 38. n_consensus_layers() now counts the
*_pts columns live from the consensus CSV header at build time, so the
copy can never go stale again; the layer-ingestion roster adds the new
families (discretionary conviction, emergence cross-feed, Sohn,
asymmetry assembly, distressed-stub, premium injections, selective
buybacks, hidden-asset realisation).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017dpaFdbqUZj62BWE6zHYXu
</commit_message>
<xml_diff>
--- a/MOST_ASYMMETRIC.xlsx
+++ b/MOST_ASYMMETRIC.xlsx
@@ -602,7 +602,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Contents — a structural map of the 30-layer universe analysis</t>
+          <t>Contents — a structural map of the 38-layer universe analysis</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -14284,10 +14284,10 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>4410</v>
+        <v>4415</v>
       </c>
       <c r="C5" s="19" t="n">
-        <v>71.54445165476963</v>
+        <v>71.62556781310838</v>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
@@ -14312,10 +14312,10 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>4410</v>
+        <v>4415</v>
       </c>
       <c r="C6" s="20" t="n">
-        <v>71.54445165476963</v>
+        <v>71.62556781310838</v>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
@@ -15787,7 +15787,7 @@
       </c>
       <c r="C6" s="25" t="inlineStr">
         <is>
-          <t>30 additive scoring layers ingested per ticker, spanning PSU forensics, governance, valuation, verified buybacks, tender mechanics, 10b5-1 direction, Form 4 (raw + Cohen-Malloy opportunistic), Form 144, quarterly 10-Q, NCAV, Voss CIC, post-Ch11, internalization, bumpitrage, spinoff timing, Arquitos, Coval-Stafford proxy + real N-PORT, backstopped rights, FDIC dark banks, activist letters, 13F-delta, biotech PDUFA, and financial-sector primary.</t>
+          <t>38 additive scoring layers ingested per ticker, spanning PSU forensics, governance, valuation, verified buybacks, tender mechanics, 10b5-1 direction, Form 4 (raw + Cohen-Malloy opportunistic), Form 144, quarterly 10-Q, NCAV, Voss CIC, post-Ch11, internalization, bumpitrage, spinoff timing, Arquitos, Coval-Stafford proxy + real N-PORT, backstopped rights, FDIC dark banks, activist letters, 13F-delta, biotech PDUFA, financial-sector primary, discretionary insider conviction, emergence cross-feed, Sohn pitches, asymmetry assembly (PSIX recipe), distressed-stub progress, premium injections, selective buybacks, and hidden-asset realisation.</t>
         </is>
       </c>
     </row>
@@ -15877,7 +15877,7 @@
       </c>
       <c r="C12" s="25" t="inlineStr">
         <is>
-          <t>Pairwise Spearman correlation (layer_correlation_pairs.csv) collapses 30 raw layers to ~21 effective-independent at rho&gt;0.6. Three correlated clusters: PSU+Voss, tender family, F4+opportunistic. 'Fires 9 layers' ≈ 7-8 true confirmations.</t>
+          <t>Pairwise Spearman correlation (layer_correlation_pairs.csv) collapses 38 raw layers to effective-independent at rho&gt;0.6. Three correlated clusters: PSU+Voss, tender family, F4+opportunistic. 'Fires 9 layers' ≈ 7-8 true confirmations.</t>
         </is>
       </c>
     </row>
@@ -19268,7 +19268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -20143,12 +20143,12 @@
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>discretionary hurdle, retirement carveout</t>
-        </is>
-      </c>
-      <c r="E40" s="10" t="inlineStr">
-        <is>
-          <t>Material — basket diversify</t>
+          <t>discretionary hurdle</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Concentrate (1 flag tolerable)</t>
         </is>
       </c>
     </row>
@@ -20250,7 +20250,7 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>PII</t>
         </is>
       </c>
       <c r="C45" s="16" t="n">
@@ -20258,12 +20258,12 @@
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>discretionary hurdle</t>
+          <t>discretionary hurdle, repricing language, retirement carveout</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Concentrate (1 flag tolerable)</t>
+          <t>Participation — limited size</t>
         </is>
       </c>
     </row>
@@ -20273,7 +20273,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>PII</t>
+          <t>TCBK</t>
         </is>
       </c>
       <c r="C46" s="17" t="n">
@@ -20296,7 +20296,7 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>TCBK</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="C47" s="16" t="n">
@@ -20304,12 +20304,12 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>discretionary hurdle, repricing language, retirement carveout</t>
+          <t>front-loaded grant</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Participation — limited size</t>
+          <t>Concentrate (1 flag tolerable)</t>
         </is>
       </c>
     </row>
@@ -20319,7 +20319,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>IDA</t>
         </is>
       </c>
       <c r="C48" s="17" t="n">
@@ -20327,7 +20327,7 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>front-loaded grant</t>
+          <t>retirement carveout</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
@@ -20342,7 +20342,7 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>IDA</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="C49" s="16" t="n">
@@ -20350,7 +20350,7 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>retirement carveout</t>
+          <t>discretionary hurdle</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -20365,7 +20365,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>SOLS</t>
         </is>
       </c>
       <c r="C50" s="17" t="n">
@@ -20373,7 +20373,7 @@
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>discretionary hurdle</t>
+          <t>retirement carveout</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
@@ -20388,7 +20388,7 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>SOLS</t>
+          <t>SIG</t>
         </is>
       </c>
       <c r="C51" s="16" t="n">
@@ -20411,7 +20411,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>SIG</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="C52" s="17" t="n">
@@ -20419,12 +20419,12 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>retirement carveout</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
-        <is>
-          <t>Concentrate (1 flag tolerable)</t>
+          <t>retirement carveout, single-trigger CIC</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>Material — basket diversify</t>
         </is>
       </c>
     </row>
@@ -20434,7 +20434,7 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>TGT</t>
+          <t>MNST</t>
         </is>
       </c>
       <c r="C53" s="16" t="n">
@@ -20442,7 +20442,7 @@
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>retirement carveout, single-trigger CIC</t>
+          <t>discretionary hurdle, retirement carveout</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
@@ -20457,7 +20457,7 @@
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>AIN</t>
         </is>
       </c>
       <c r="C54" s="17" t="n">
@@ -20465,12 +20465,12 @@
       </c>
       <c r="D54" s="10" t="inlineStr">
         <is>
-          <t>discretionary hurdle, retirement carveout</t>
-        </is>
-      </c>
-      <c r="E54" s="10" t="inlineStr">
-        <is>
-          <t>Material — basket diversify</t>
+          <t>retirement carveout</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>Concentrate (1 flag tolerable)</t>
         </is>
       </c>
     </row>
@@ -20480,7 +20480,7 @@
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>AIN</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="C55" s="16" t="n">
@@ -20488,7 +20488,7 @@
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>discretionary hurdle, retirement carveout</t>
+          <t>repricing language, retirement carveout</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
@@ -20503,7 +20503,7 @@
       </c>
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>IDCC</t>
         </is>
       </c>
       <c r="C56" s="17" t="n">
@@ -20511,7 +20511,7 @@
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>repricing language, retirement carveout</t>
+          <t>retirement carveout, single-trigger CIC</t>
         </is>
       </c>
       <c r="E56" s="10" t="inlineStr">
@@ -20526,7 +20526,7 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>IDCC</t>
+          <t>MERC</t>
         </is>
       </c>
       <c r="C57" s="16" t="n">
@@ -20534,7 +20534,7 @@
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>retirement carveout, single-trigger CIC</t>
+          <t>discretionary hurdle, retirement carveout</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
@@ -20549,7 +20549,7 @@
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>MERC</t>
+          <t>ACH</t>
         </is>
       </c>
       <c r="C58" s="17" t="n">
@@ -20557,7 +20557,7 @@
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>discretionary hurdle, retirement carveout</t>
+          <t>discretionary hurdle, front-loaded grant</t>
         </is>
       </c>
       <c r="E58" s="10" t="inlineStr">
@@ -20572,7 +20572,7 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>ACH</t>
+          <t>BUSE</t>
         </is>
       </c>
       <c r="C59" s="16" t="n">
@@ -20580,12 +20580,12 @@
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>discretionary hurdle, front-loaded grant</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="inlineStr">
-        <is>
-          <t>Material — basket diversify</t>
+          <t>retirement carveout</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Concentrate (1 flag tolerable)</t>
         </is>
       </c>
     </row>
@@ -20595,7 +20595,7 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>BUSE</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="C60" s="17" t="n">
@@ -20603,40 +20603,17 @@
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>retirement carveout</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>Concentrate (1 flag tolerable)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="30" customHeight="1">
-      <c r="A61" s="5" t="n">
-        <v>57</v>
-      </c>
-      <c r="B61" s="6" t="inlineStr">
-        <is>
-          <t>NXT</t>
-        </is>
-      </c>
-      <c r="C61" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="D61" s="7" t="inlineStr">
-        <is>
           <t>repricing language, retirement carveout</t>
         </is>
       </c>
-      <c r="E61" s="7" t="inlineStr">
+      <c r="E60" s="10" t="inlineStr">
         <is>
           <t>Material — basket diversify</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="28" customHeight="1">
-      <c r="A63" s="11" t="inlineStr">
+    <row r="62" ht="28" customHeight="1">
+      <c r="A62" s="11" t="inlineStr">
         <is>
           <t>Eight flag classes: single-trigger CIC, repricing language, retirement carveout, front-loaded grant, discretionary hurdle, aggregate-only metrics, plus structural variants. Counter-intuitive: a 'repricing language' flag can become a re-rate catalyst when a stock has fallen sharply, since management becomes incentivised to reset hurdles. Read the flag in context, not as automatic veto.</t>
         </is>
@@ -20646,7 +20623,7 @@
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A63:E63"/>
+    <mergeCell ref="A62:E62"/>
   </mergeCells>
   <printOptions horizontalCentered="0"/>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
@@ -20784,400 +20761,404 @@
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>AGNC</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>DocuSign, Inc.</t>
+          <t>AGNC Investment Corp.</t>
         </is>
       </c>
       <c r="C6" s="17" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>34</v>
+        <v>3.8</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F6" s="20" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="G6" s="17" t="n">
-        <v>4.6117125</v>
+        <v>1.1440774</v>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>PSU weight increased; shareholder-responsive redesign; vesting period extended</t>
+          <t>PSU weight increased; shareholder-responsive redesign; clawback strengthened</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>front-loaded grant (worse) · 2026-04-16</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>CMLSQ</t>
+          <t>AGNCL</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Cumulus Media Inc.</t>
+          <t>AGNCL</t>
         </is>
       </c>
       <c r="C7" s="16" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-4</v>
+        <v>4</v>
       </c>
       <c r="F7" s="19" t="n">
-        <v>30</v>
-      </c>
-      <c r="G7" s="16" t="n">
-        <v>-0.0003314917</v>
+        <v>50</v>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>ownership requirement added; shareholder-responsive redesign; clawback strengthened; follo</t>
+          <t>PSU weight increased; shareholder-responsive redesign; clawback strengthened</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>2025-04-25</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>AIG</t>
+          <t>AGNCM</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>American International Gro</t>
+          <t>AGNCM</t>
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>10.5</v>
+        <v>3.8</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G8" s="17" t="n">
-        <v>0.9762594999999999</v>
+        <v>4</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>new performance metric; PSU weight increased</t>
+          <t>PSU weight increased; shareholder-responsive redesign; clawback strengthened</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>GFF</t>
+          <t>AGNCN</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Griffon Corporation</t>
+          <t>AGNCN</t>
         </is>
       </c>
       <c r="C9" s="16" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>37.5</v>
+        <v>3.8</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G9" s="16" t="n">
-        <v>44.497066</v>
+        <v>4</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>50</v>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>new performance metric; shareholder-responsive redesign; clawback strengthened; anti-hedge</t>
+          <t>PSU weight increased; shareholder-responsive redesign; clawback strengthened</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>COUR</t>
+          <t>AGNCO</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Coursera, Inc.</t>
+          <t>AGNCO</t>
         </is>
       </c>
       <c r="C10" s="17" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>30.6</v>
+        <v>3.8</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="G10" s="17" t="n">
-        <v>1.4335476</v>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>PSU weight increased; anti-hedge/pledge added; follows SOP dissent (60%)</t>
+          <t>PSU weight increased; shareholder-responsive redesign; clawback strengthened</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>EHTH</t>
+          <t>AGNCP</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>eHealth, Inc.</t>
+          <t>AGNCP</t>
         </is>
       </c>
       <c r="C11" s="16" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>21.6</v>
+        <v>3.8</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="n">
-        <v>0.08644627000000001</v>
+        <v>4</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>50</v>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>PSU weight increased; vesting period extended</t>
+          <t>PSU weight increased; shareholder-responsive redesign; clawback strengthened</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-03-06</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>IQV</t>
+          <t>DOCU</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>IQVIA Holdings, Inc.</t>
+          <t>DocuSign, Inc.</t>
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>-7</v>
-      </c>
-      <c r="F12" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="F12" s="20" t="n">
+        <v>60</v>
       </c>
       <c r="G12" s="17" t="n">
-        <v>4.996781</v>
+        <v>4.6117125</v>
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>PSU weight increased; clawback strengthened; follows SOP dissent (65%)</t>
+          <t>PSU weight increased; shareholder-responsive redesign; vesting period extended</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>front-loaded grant (worse) · 2026-04-16</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>BILL</t>
+          <t>CMLSQ</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>BILL Holdings, Inc.</t>
+          <t>Cumulus Media Inc.</t>
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>29.4</v>
+        <v>0</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>15</v>
+        <v>-4</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>0.8502894</v>
+        <v>-0.0003314917</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>PSU weight increased; shareholder-responsive redesign</t>
+          <t>ownership requirement added; shareholder-responsive redesign; clawback strengthened; follo</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>2025-10-27</t>
+          <t>2025-04-25</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>UPWK</t>
+          <t>AIG</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Upwork Inc.</t>
+          <t>American International Gro</t>
         </is>
       </c>
       <c r="C14" s="17" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>39.6</v>
+        <v>10.5</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="F14" s="20" t="n">
-        <v>60</v>
+        <v>2</v>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G14" s="17" t="n">
-        <v>1.7462039</v>
+        <v>0.9762594999999999</v>
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>PSU weight increased; shareholder-responsive redesign</t>
+          <t>new performance metric; PSU weight increased</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>DCH</t>
+          <t>AMT</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Dauch Corporation</t>
+          <t>American Tower Corporation</t>
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>47.7</v>
+        <v>42</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>0.9973131</v>
+        <v>23.290117</v>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>PSU weight increased; shareholder-responsive redesign</t>
+          <t>new performance metric; PSU weight increased</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>SMHI</t>
+          <t>GFF</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>SEACOR Marine Holdings Inc</t>
+          <t>Griffon Corporation</t>
         </is>
       </c>
       <c r="C16" s="17" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>15</v>
+        <v>37.5</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
@@ -21185,75 +21166,75 @@
         </is>
       </c>
       <c r="G16" s="17" t="n">
-        <v>0.7303739</v>
+        <v>44.497066</v>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>clawback strengthened; anti-hedge/pledge added; vesting period extended; follows SOP disse</t>
+          <t>new performance metric; shareholder-responsive redesign; clawback strengthened; anti-hedge</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-01-09</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>COUR</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Intercontinental Exchange</t>
+          <t>Coursera, Inc.</t>
         </is>
       </c>
       <c r="C17" s="16" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>23.4</v>
+        <v>30.6</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="G17" s="16" t="n">
-        <v>2.5706112</v>
+        <v>1.4335476</v>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added; follows S</t>
+          <t>PSU weight increased; anti-hedge/pledge added; follows SOP dissent (60%)</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-05-11</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>CGNX</t>
+          <t>EHTH</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Cognex Corporation</t>
+          <t>eHealth, Inc.</t>
         </is>
       </c>
       <c r="C18" s="17" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>12.6</v>
+        <v>21.6</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
@@ -21261,186 +21242,188 @@
         </is>
       </c>
       <c r="G18" s="17" t="n">
-        <v>7.442856</v>
+        <v>0.08644627000000001</v>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added; follows S</t>
+          <t>PSU weight increased; vesting period extended</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-04-28</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>IQV</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>SentinelOne, Inc.</t>
+          <t>IQVIA Holdings, Inc.</t>
         </is>
       </c>
       <c r="C19" s="16" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="19" t="n">
-        <v>50</v>
+        <v>-7</v>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G19" s="16" t="n">
-        <v>3.5299647</v>
+        <v>4.996781</v>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>PSU weight increased; anti-hedge/pledge added</t>
+          <t>PSU weight increased; clawback strengthened; follows SOP dissent (65%)</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-02-27</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>BURL</t>
+          <t>BILL</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Burlington Stores, Inc.</t>
+          <t>BILL Holdings, Inc.</t>
         </is>
       </c>
       <c r="C20" s="17" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>9.9</v>
+        <v>29.4</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="F20" s="20" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="G20" s="17" t="n">
-        <v>11.411977</v>
+        <v>0.8502894</v>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>PSU weight increased; anti-hedge/pledge added</t>
+          <t>PSU weight increased; shareholder-responsive redesign</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2025-10-27</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>THRY</t>
+          <t>UPWK</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Thryv Holdings, Inc.</t>
+          <t>Upwork Inc.</t>
         </is>
       </c>
       <c r="C21" s="16" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>11.7</v>
+        <v>39.6</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F21" s="19" t="n">
         <v>60</v>
       </c>
       <c r="G21" s="16" t="n">
-        <v>0.6885697</v>
+        <v>1.7462039</v>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>ownership requirement added; clawback strengthened; anti-hedge/pledge added</t>
+          <t>PSU weight increased; shareholder-responsive redesign</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>BFH</t>
+          <t>DCH</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Bread Financial Holdings,</t>
+          <t>Dauch Corporation</t>
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>30.8</v>
+        <v>47.7</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F22" s="20" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="G22" s="17" t="n">
-        <v>1.2720475</v>
+        <v>0.9973131</v>
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>new performance metric; clawback strengthened; anti-hedge/pledge added</t>
+          <t>PSU weight increased; shareholder-responsive redesign</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>UPST</t>
+          <t>SMHI</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Upstart Holdings, Inc.</t>
+          <t>SEACOR Marine Holdings Inc</t>
         </is>
       </c>
       <c r="C23" s="16" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>6.8</v>
+        <v>15</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -21448,11 +21431,11 @@
         </is>
       </c>
       <c r="G23" s="16" t="n">
-        <v>4.2336817</v>
+        <v>0.7303739</v>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>new performance metric; anti-hedge/pledge added; follows SOP dissent (74%)</t>
+          <t>clawback strengthened; anti-hedge/pledge added; vesting period extended; follows SOP disse</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
@@ -21464,69 +21447,71 @@
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>MUR</t>
+          <t>AMN</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Murphy Oil Corporation</t>
+          <t>AMN Healthcare Services In</t>
         </is>
       </c>
       <c r="C24" s="17" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>11.2</v>
+        <v>38.2</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="F24" s="20" t="n">
-        <v>80</v>
+        <v>11</v>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G24" s="17" t="n">
-        <v>0.96401465</v>
+        <v>1.6801345</v>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>new performance metric; anti-hedge/pledge added; follows SOP dissent (40%)</t>
+          <t>new performance metric; shareholder-responsive redesign; follows SOP dissent (78%)</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-18</t>
         </is>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>CORZ</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Core Scientific, Inc.</t>
+          <t>Intercontinental Exchange</t>
         </is>
       </c>
       <c r="C25" s="16" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>12.6</v>
+        <v>23.4</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="F25" s="19" t="n">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="G25" s="16" t="n">
-        <v>-7.07767</v>
+        <v>2.5706112</v>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>PSU weight increased; follows SOP dissent (38%)</t>
+          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added; follows S</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
@@ -21538,22 +21523,22 @@
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>ONIT</t>
+          <t>CGNX</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Onity Group Inc.</t>
+          <t>Cognex Corporation</t>
         </is>
       </c>
       <c r="C26" s="17" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>21.8</v>
+        <v>12.6</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
@@ -21561,574 +21546,572 @@
         </is>
       </c>
       <c r="G26" s="17" t="n">
-        <v>0.4901751</v>
+        <v>7.442856</v>
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>new performance metric; clawback strengthened; follows SOP dissent (76%)</t>
+          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added; follows S</t>
         </is>
       </c>
       <c r="I26" s="10" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>ATEN</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>A10 Networks, Inc.</t>
+          <t>SentinelOne, Inc.</t>
         </is>
       </c>
       <c r="C27" s="16" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>30.6</v>
+        <v>15</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="F27" s="19" t="n">
         <v>50</v>
       </c>
       <c r="G27" s="16" t="n">
-        <v>10.80923</v>
+        <v>3.5299647</v>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>clawback strengthened; anti-hedge/pledge added; vesting period extended</t>
+          <t>PSU weight increased; anti-hedge/pledge added</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>BURL</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>JFrog Ltd.</t>
+          <t>Burlington Stores, Inc.</t>
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>29.7</v>
+        <v>9.9</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>-6</v>
+        <v>1</v>
       </c>
       <c r="F28" s="20" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="G28" s="17" t="n">
-        <v>10.847102</v>
+        <v>11.411977</v>
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>ownership requirement added; vesting period extended</t>
+          <t>PSU weight increased; anti-hedge/pledge added</t>
         </is>
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-02</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>THRY</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Agilent Technologies, Inc.</t>
+          <t>Thryv Holdings, Inc.</t>
         </is>
       </c>
       <c r="C29" s="16" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>39.8</v>
+        <v>11.7</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F29" s="19" t="n">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="G29" s="16" t="n">
-        <v>5.0348706</v>
+        <v>0.6885697</v>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
+          <t>ownership requirement added; clawback strengthened; anti-hedge/pledge added</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>CNC</t>
+          <t>BFH</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Centene Corporation</t>
+          <t>Bread Financial Holdings,</t>
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>19.8</v>
+        <v>30.8</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="F30" s="20" t="n">
         <v>60</v>
       </c>
       <c r="G30" s="17" t="n">
-        <v>1.4061527</v>
+        <v>1.2720475</v>
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
+          <t>new performance metric; clawback strengthened; anti-hedge/pledge added</t>
         </is>
       </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>ADC</t>
+          <t>UPST</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Agree Realty Corporation</t>
+          <t>Upstart Holdings, Inc.</t>
         </is>
       </c>
       <c r="C31" s="16" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>2.7</v>
+        <v>6.8</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="19" t="n">
-        <v>45</v>
+        <v>7</v>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G31" s="16" t="n">
-        <v>1.4485731</v>
+        <v>4.2336817</v>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>ownership requirement added; shareholder-responsive redesign</t>
+          <t>new performance metric; anti-hedge/pledge added; follows SOP dissent (74%)</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>IRTC</t>
+          <t>MUR</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>iRhythm Holdings, Inc.</t>
+          <t>Murphy Oil Corporation</t>
         </is>
       </c>
       <c r="C32" s="17" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>28</v>
+        <v>11.2</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F32" s="20" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G32" s="17" t="n">
-        <v>21.326675</v>
+        <v>0.96401465</v>
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t>ownership requirement added; shareholder-responsive redesign</t>
+          <t>new performance metric; anti-hedge/pledge added; follows SOP dissent (40%)</t>
         </is>
       </c>
       <c r="I32" s="10" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-03-27</t>
         </is>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>LC</t>
+          <t>ASTE</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>LendingClub Corporation</t>
+          <t>Astec Industries, Inc.</t>
         </is>
       </c>
       <c r="C33" s="16" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="F33" s="19" t="n">
+        <v>65</v>
       </c>
       <c r="G33" s="16" t="n">
-        <v>1.4771241</v>
+        <v>1.901406</v>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
+          <t>PSU weight increased; clawback strengthened</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>NTGR</t>
+          <t>CORZ</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>NETGEAR, Inc.</t>
+          <t>Core Scientific, Inc.</t>
         </is>
       </c>
       <c r="C34" s="17" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>26</v>
+        <v>12.6</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F34" s="20" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G34" s="17" t="n">
-        <v>1.3377051</v>
+        <v>-7.07767</v>
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
+          <t>PSU weight increased; follows SOP dissent (38%)</t>
         </is>
       </c>
       <c r="I34" s="10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-03-31</t>
         </is>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>ONIT</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>Onity Group Inc.</t>
         </is>
       </c>
       <c r="C35" s="16" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>0</v>
+        <v>21.8</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="F35" s="19" t="n">
-        <v>25</v>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>11</v>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G35" s="16" t="n">
+        <v>0.4901751</v>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
+          <t>new performance metric; clawback strengthened; follows SOP dissent (76%)</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-14</t>
         </is>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>ATEN</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>Lithia Motors, Inc.</t>
+          <t>A10 Networks, Inc.</t>
         </is>
       </c>
       <c r="C36" s="17" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="F36" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>19</v>
+      </c>
+      <c r="F36" s="20" t="n">
+        <v>50</v>
       </c>
       <c r="G36" s="17" t="n">
-        <v>1.0530019</v>
+        <v>10.80923</v>
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>clawback strengthened; vesting period extended; follows SOP dissent (45%)</t>
+          <t>clawback strengthened; anti-hedge/pledge added; vesting period extended</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-10</t>
         </is>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>CSGP</t>
+          <t>FROG</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>CoStar Group, Inc.</t>
+          <t>JFrog Ltd.</t>
         </is>
       </c>
       <c r="C37" s="16" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D37" s="5" t="n">
-        <v>40.5</v>
+        <v>29.7</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>14</v>
+        <v>-6</v>
       </c>
       <c r="F37" s="19" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="G37" s="16" t="n">
-        <v>1.5496218</v>
+        <v>10.847102</v>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; follows SOP dissent (53%)</t>
+          <t>ownership requirement added; vesting period extended</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-07</t>
         </is>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>IHRT</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>iHeartMedia, Inc.</t>
+          <t>Agilent Technologies, Inc.</t>
         </is>
       </c>
       <c r="C38" s="17" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="F38" s="20" t="n">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="G38" s="17" t="n">
-        <v>-0.32349604</v>
+        <v>5.0348706</v>
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; follows SOP dissent (73%)</t>
+          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
         </is>
       </c>
       <c r="I38" s="10" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-02-06</t>
         </is>
       </c>
     </row>
     <row r="39" ht="24" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>PTN</t>
+          <t>AMCX</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Palatin Technologies, Inc.</t>
+          <t>AMC Global Media Inc.</t>
         </is>
       </c>
       <c r="C39" s="16" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D39" s="5" t="n">
-        <v>20.4</v>
+        <v>5.4</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F39" s="19" t="n">
-        <v>50</v>
+        <v>7</v>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G39" s="16" t="n">
-        <v>1.9654537</v>
+        <v>0.43042397</v>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; follows SOP dissent (58%)</t>
+          <t>new performance metric; shareholder-responsive redesign</t>
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>2025-06-30</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
     <row r="40" ht="24" customHeight="1">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>CNC</t>
         </is>
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Vaxcyte, Inc.</t>
+          <t>Centene Corporation</t>
         </is>
       </c>
       <c r="C40" s="17" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>12</v>
+        <v>19.8</v>
       </c>
       <c r="E40" s="8" t="n">
-        <v>-4</v>
+        <v>7</v>
       </c>
       <c r="F40" s="20" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G40" s="17" t="n">
-        <v>2.4778419</v>
+        <v>1.4061527</v>
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; follows SOP dissent (64%)</t>
+          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
         </is>
       </c>
       <c r="I40" s="10" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-03-26</t>
         </is>
       </c>
     </row>
     <row r="41" ht="24" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>PSX</t>
+          <t>ADC</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Phillips 66</t>
+          <t>Agree Realty Corporation</t>
         </is>
       </c>
       <c r="C41" s="16" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D41" s="5" t="n">
-        <v>18</v>
+        <v>2.7</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="F41" s="19" t="n">
+        <v>45</v>
       </c>
       <c r="G41" s="16" t="n">
-        <v>2.3349354</v>
+        <v>1.4485731</v>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; vesting period extended</t>
+          <t>ownership requirement added; shareholder-responsive redesign</t>
         </is>
       </c>
       <c r="I41" s="7" t="inlineStr">
@@ -22140,170 +22123,174 @@
     <row r="42" ht="24" customHeight="1">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>SHLS</t>
+          <t>IRTC</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Shoals Technologies Group,</t>
+          <t>iRhythm Holdings, Inc.</t>
         </is>
       </c>
       <c r="C42" s="17" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D42" s="8" t="n">
-        <v>19.8</v>
+        <v>28</v>
       </c>
       <c r="E42" s="8" t="n">
-        <v>-4</v>
+        <v>1</v>
       </c>
       <c r="F42" s="20" t="n">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="G42" s="17" t="n">
-        <v>2.9057446</v>
+        <v>21.326675</v>
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>shareholder-responsive redesign; clawback strengthened; follows SOP dissent (61%)</t>
+          <t>ownership requirement added; shareholder-responsive redesign</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
         <is>
-          <t>2026-03-20</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
     <row r="43" ht="24" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>VITL</t>
+          <t>LC</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Vital Farms, Inc.</t>
+          <t>LendingClub Corporation</t>
         </is>
       </c>
       <c r="C43" s="16" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D43" s="5" t="n">
-        <v>26.1</v>
+        <v>11</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="F43" s="19" t="n">
-        <v>50</v>
+        <v>13</v>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G43" s="16" t="n">
-        <v>1.3276367</v>
+        <v>1.4771241</v>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>ownership requirement added; anti-hedge/pledge added</t>
+          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
         </is>
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-21</t>
         </is>
       </c>
     </row>
     <row r="44" ht="24" customHeight="1">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>NTGR</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>Grocery Outlet Holding Cor</t>
+          <t>NETGEAR, Inc.</t>
         </is>
       </c>
       <c r="C44" s="17" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>69.3</v>
+        <v>26</v>
       </c>
       <c r="E44" s="8" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F44" s="20" t="n">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="G44" s="17" t="n">
-        <v>1.134943</v>
+        <v>1.3377051</v>
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>PSU weight increased</t>
+          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
         </is>
       </c>
       <c r="I44" s="10" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
     <row r="45" ht="24" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>KHC</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>The Kraft Heinz Company</t>
+          <t>SSNC</t>
         </is>
       </c>
       <c r="C45" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="F45" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="D45" s="5" t="n">
-        <v>36.8</v>
-      </c>
-      <c r="E45" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F45" s="19" t="n">
-        <v>75</v>
-      </c>
-      <c r="G45" s="16" t="n">
-        <v>0.64558107</v>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>PSU weight increased</t>
+          <t>shareholder-responsive redesign; clawback strengthened; anti-hedge/pledge added</t>
         </is>
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-08</t>
         </is>
       </c>
     </row>
     <row r="46" ht="24" customHeight="1">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>IONS</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>Ionis Pharmaceuticals, Inc</t>
+          <t>Lithia Motors, Inc.</t>
         </is>
       </c>
       <c r="C46" s="17" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D46" s="8" t="n">
-        <v>27.9</v>
+        <v>9</v>
       </c>
       <c r="E46" s="8" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F46" s="10" t="inlineStr">
         <is>
@@ -22311,136 +22298,134 @@
         </is>
       </c>
       <c r="G46" s="17" t="n">
-        <v>25.023634</v>
+        <v>1.0530019</v>
       </c>
       <c r="H46" s="10" t="inlineStr">
         <is>
-          <t>PSU weight increased</t>
+          <t>clawback strengthened; vesting period extended; follows SOP dissent (45%)</t>
         </is>
       </c>
       <c r="I46" s="10" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-03-11</t>
         </is>
       </c>
     </row>
     <row r="47" ht="24" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>SPCE</t>
+          <t>CSGP</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Virgin Galactic Holdings,</t>
+          <t>CoStar Group, Inc.</t>
         </is>
       </c>
       <c r="C47" s="16" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>25.2</v>
+        <v>40.5</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F47" s="19" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G47" s="16" t="n">
-        <v>1.2954876</v>
+        <v>1.5496218</v>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>PSU weight increased</t>
+          <t>shareholder-responsive redesign; clawback strengthened; follows SOP dissent (53%)</t>
         </is>
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-30</t>
         </is>
       </c>
     </row>
     <row r="48" ht="24" customHeight="1">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>CHD</t>
+          <t>IHRT</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Church &amp; Dwight Company, I</t>
+          <t>iHeartMedia, Inc.</t>
         </is>
       </c>
       <c r="C48" s="17" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D48" s="8" t="n">
-        <v>8.1</v>
+        <v>0</v>
       </c>
       <c r="E48" s="8" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F48" s="20" t="n">
         <v>50</v>
       </c>
       <c r="G48" s="17" t="n">
-        <v>5.4116917</v>
+        <v>-0.32349604</v>
       </c>
       <c r="H48" s="10" t="inlineStr">
         <is>
-          <t>PSU weight increased</t>
+          <t>shareholder-responsive redesign; clawback strengthened; follows SOP dissent (73%)</t>
         </is>
       </c>
       <c r="I48" s="10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-04-17</t>
         </is>
       </c>
     </row>
     <row r="49" ht="24" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>PTN</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>PTC Inc.</t>
+          <t>Palatin Technologies, Inc.</t>
         </is>
       </c>
       <c r="C49" s="16" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D49" s="5" t="n">
-        <v>9.800000000000001</v>
+        <v>20.4</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>6</v>
+      </c>
+      <c r="F49" s="19" t="n">
+        <v>50</v>
       </c>
       <c r="G49" s="16" t="n">
-        <v>3.4336755</v>
+        <v>1.9654537</v>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>PSU weight increased</t>
+          <t>shareholder-responsive redesign; clawback strengthened; follows SOP dissent (58%)</t>
         </is>
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>2025-12-23</t>
+          <t>2025-06-30</t>
         </is>
       </c>
     </row>
     <row r="51" ht="28" customHeight="1">
       <c r="A51" s="11" t="inlineStr">
         <is>
-          <t>992 names show at least one structural improvement in the latest proxy (top 45 shown). Weights reflect rarity across 4,410 scanned DEF 14As: PSU-weight increase (12 occurrences, +25) and ownership-requirement addition (23, +15) are deliberate alignment choices; clawback strengthening (607, +4) and anti-hedge language (331, +6) are largely post-2023 SEC-rule boilerplate. Multi-improvement redesigns earn a conjunction bonus; improvements that follow a sub-80% say-on-pay vote are tagged as forced-response. Regressions (front-loaded grants, metric elimination) subtract and are listed as caveats. Source: proxy_scan plan_deltas + pattern_reasons -- fully data-driven.</t>
+          <t>999 names show at least one structural improvement in the latest proxy (top 45 shown). Weights reflect rarity across 4,410 scanned DEF 14As: PSU-weight increase (12 occurrences, +25) and ownership-requirement addition (23, +15) are deliberate alignment choices; clawback strengthening (607, +4) and anti-hedge language (331, +6) are largely post-2023 SEC-rule boilerplate. Multi-improvement redesigns earn a conjunction bonus; improvements that follow a sub-80% say-on-pay vote are tagged as forced-response. Regressions (front-loaded grants, metric elimination) subtract and are listed as caveats. Source: proxy_scan plan_deltas + pattern_reasons -- fully data-driven.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Full derived rebuild on improved code (39 layers, frames store, decay, health gate)
Regenerated every deliverable over the current engine: consensus (39
scoring layers incl. equity_committee + all revealed-preference /
distressed / hidden-asset legs), catalyst decay applied, frames-store-fed
assembly, rankers, correlation, SYSTEMATIC_RANKINGS, and MOST_ASYMMETRIC
(20 tabs). Source-health gate: all 20 consumed sources OK. Tests green.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017dpaFdbqUZj62BWE6zHYXu
</commit_message>
<xml_diff>
--- a/MOST_ASYMMETRIC.xlsx
+++ b/MOST_ASYMMETRIC.xlsx
@@ -605,7 +605,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Contents — a structural map of the 38-layer universe analysis</t>
+          <t>Contents — a structural map of the 39-layer universe analysis</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -4274,10 +4274,10 @@
         <v>8</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>6.154</v>
+        <v>5.902</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -4296,22 +4296,22 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>FOUR</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Shift4 Payments, Inc.</t>
+          <t>Salesforce, Inc.</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>6.012</v>
+        <v>5.764</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
@@ -4320,7 +4320,7 @@
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>PSU:28 BB:5 F4:10 RI:51</t>
+          <t>PSU:28 BB:8 C10:-5 F4:11 RI:61</t>
         </is>
       </c>
     </row>
@@ -4342,7 +4342,7 @@
         <v>7</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>5.986</v>
+        <v>5.626</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-2</v>
@@ -4364,22 +4364,22 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>HubSpot, Inc.</t>
+          <t>PAR Technology Corporation</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>5.826</v>
+        <v>5.546</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>PSU:25 BB:5 F4:17 RI:57</t>
+          <t>PSU:17 C10:-50 RI:45 SS:35</t>
         </is>
       </c>
     </row>
@@ -4398,22 +4398,24 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>FOUR</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Salesforce, Inc.</t>
+          <t>Shift4 Payments, Inc.</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
         <v>7</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>5.684</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>-2</v>
+        <v>5.478</v>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
@@ -4422,7 +4424,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>PSU:28 BB:8 C10:-5 F4:11 RI:61</t>
+          <t>PSU:28 BB:5 F4:10 RI:51</t>
         </is>
       </c>
     </row>
@@ -4432,22 +4434,22 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Universal Display Corporation</t>
+          <t>HubSpot, Inc.</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>5.302</v>
+        <v>5.452</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
@@ -4456,7 +4458,7 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>PSU:40 BB:5 F4:17 RI:60</t>
+          <t>PSU:25 BB:5 F4:17 RI:57</t>
         </is>
       </c>
     </row>
@@ -4466,22 +4468,22 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>DXC</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>DXC Technology Company</t>
+          <t>Universal Display Corporation</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
         <v>7</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>5.044</v>
+        <v>5.378</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-3</v>
+        <v>4</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
@@ -4490,7 +4492,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>PSU:43 BB:5 RI:57</t>
+          <t>PSU:40 BB:5 F4:17 RI:60</t>
         </is>
       </c>
     </row>
@@ -4500,22 +4502,22 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>BLND</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>PAR Technology Corporation</t>
+          <t>Blend Labs, Inc.</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>4.994</v>
+        <v>4.808</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>-2</v>
+        <v>17</v>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
@@ -4524,7 +4526,7 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>PSU:17 C10:-50 RI:45 SS:35</t>
+          <t>PSU:8 BB:5 C10:-35 F4:5 RI:52 SS:20</t>
         </is>
       </c>
     </row>
@@ -4534,31 +4536,31 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>BLND</t>
+          <t>ADT</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Blend Labs, Inc.</t>
+          <t>ADT Inc.</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
         <v>7</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>4.946</v>
+        <v>4.59</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>12</v>
+        <v>-1</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>PSU:8 BB:5 C10:-35 F4:5 RI:52 SS:20</t>
+          <t>PSU:31 BB:5 F4:12 RI:50 SS:10</t>
         </is>
       </c>
     </row>
@@ -4580,10 +4582,10 @@
         <v>7</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>4.318</v>
+        <v>4.514</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
@@ -4602,31 +4604,31 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>CERT</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>ADT Inc.</t>
+          <t>Certara, Inc.</t>
         </is>
       </c>
       <c r="D15" s="5" t="n">
         <v>7</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>4.28</v>
+        <v>4.416</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-3</v>
+        <v>17</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>PSU:31 BB:5 F4:12 RI:50 SS:10</t>
+          <t>PSU:29 BB:5 C10:-12 RI:43</t>
         </is>
       </c>
     </row>
@@ -4636,31 +4638,31 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>VTS</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>Certara, Inc.</t>
+          <t>Vitesse Energy, Inc.</t>
         </is>
       </c>
       <c r="D16" s="8" t="n">
         <v>7</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>4.094</v>
+        <v>4.12</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>14</v>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>PSU:29 BB:5 C10:-12 RI:43</t>
+          <t>PSU:28 F4:5 RI:50</t>
         </is>
       </c>
     </row>
@@ -4682,10 +4684,10 @@
         <v>6</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>5.518</v>
+        <v>5.384</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
@@ -4704,31 +4706,31 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>HDSN</t>
+          <t>SBET</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Hudson Technologies, Inc.</t>
+          <t>SharpLink, Inc.</t>
         </is>
       </c>
       <c r="D18" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>4.87</v>
+        <v>4.866</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>BB:5 F4:18 RI:58</t>
+          <t>PSU:19 C10:15 RI:71</t>
         </is>
       </c>
     </row>
@@ -4738,31 +4740,33 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>SBET</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>SharpLink, Inc.</t>
+          <t>DXC Technology Company</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>4.856</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>19</v>
+        <v>4.82</v>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>PSU:19 C10:15 RI:71</t>
+          <t>PSU:43 BB:5 RI:57</t>
         </is>
       </c>
     </row>
@@ -4772,31 +4776,31 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>ALKT</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Zoetis Inc.</t>
+          <t>Alkami Technology, Inc.</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>4.814</v>
+        <v>4.816</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>PSU:7 BB:5 C10:-3 F4:12 RI:60</t>
+          <t>PSU:11 C10:-6 F4:16 RI:54</t>
         </is>
       </c>
     </row>
@@ -4806,31 +4810,31 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>SNBR</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Sleep Number Corporation</t>
+          <t>GPGI, Inc.</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E21" s="16" t="n">
-        <v>4.742</v>
+        <v>4.762</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>PSU:49 RI:46 SS:20</t>
+          <t>PSU:17 C10:-15 F4:12 RI:52 SS:23</t>
         </is>
       </c>
     </row>
@@ -4840,31 +4844,31 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>NUS</t>
+          <t>SNBR</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Nu Skin Enterprises, Inc.</t>
+          <t>Sleep Number Corporation</t>
         </is>
       </c>
       <c r="D22" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>4.734</v>
+        <v>4.742</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>13</v>
+        <v>-6</v>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>Consumer Defensive</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>PSU:54 BB:5 C10:-32 RI:53</t>
+          <t>PSU:49 RI:46 SS:20</t>
         </is>
       </c>
     </row>
@@ -4874,31 +4878,31 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>ALKT</t>
+          <t>ACM</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Alkami Technology, Inc.</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E23" s="16" t="n">
-        <v>4.732</v>
+        <v>4.68</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>PSU:11 C10:-6 F4:16 RI:54</t>
+          <t>BB:5 F4:6 RI:54</t>
         </is>
       </c>
     </row>
@@ -4908,31 +4912,31 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>HDSN</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>GPGI, Inc.</t>
+          <t>Hudson Technologies, Inc.</t>
         </is>
       </c>
       <c r="D24" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>4.592</v>
+        <v>4.66</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>PSU:17 C10:-15 F4:12 RI:52 SS:23</t>
+          <t>BB:5 F4:18 RI:58</t>
         </is>
       </c>
     </row>
@@ -4942,31 +4946,31 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>MSCI</t>
+          <t>NUS</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>MSCI Inc.</t>
+          <t>Nu Skin Enterprises, Inc.</t>
         </is>
       </c>
       <c r="D25" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E25" s="16" t="n">
-        <v>4.56</v>
+        <v>4.562</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Consumer Defensive</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>PSU:36 BB:8 C10:-26 F4:16 RI:16</t>
+          <t>PSU:54 BB:5 C10:-32 RI:53</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4992,7 @@
         <v>6</v>
       </c>
       <c r="E26" s="17" t="n">
-        <v>4.554</v>
+        <v>4.556</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>-9</v>
@@ -5010,22 +5014,22 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>ZTS</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Option Care Health, Inc.</t>
+          <t>Zoetis Inc.</t>
         </is>
       </c>
       <c r="D27" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E27" s="16" t="n">
-        <v>4.448</v>
+        <v>4.522</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
@@ -5034,7 +5038,7 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>PSU:27 BB:5 C10:-1 F4:23 RI:52</t>
+          <t>PSU:7 BB:5 C10:-3 F4:12 RI:60</t>
         </is>
       </c>
     </row>
@@ -5044,31 +5048,31 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>MSCI</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Azenta, Inc.</t>
+          <t>MSCI Inc.</t>
         </is>
       </c>
       <c r="D28" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E28" s="17" t="n">
-        <v>4.254</v>
+        <v>4.498</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>-1</v>
+        <v>14</v>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>PSU:31</t>
+          <t>PSU:36 BB:8 C10:-26 F4:16 RI:16</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5094,7 @@
         <v>6</v>
       </c>
       <c r="E29" s="16" t="n">
-        <v>4.038</v>
+        <v>4.466</v>
       </c>
       <c r="F29" s="5" t="n">
         <v>16</v>
@@ -5112,31 +5116,31 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>ACM</t>
+          <t>AZTA</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>Azenta, Inc.</t>
         </is>
       </c>
       <c r="D30" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E30" s="17" t="n">
-        <v>3.992</v>
+        <v>4.348</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>20</v>
+        <v>-3</v>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>BB:5 F4:6 RI:54</t>
+          <t>PSU:31</t>
         </is>
       </c>
     </row>
@@ -5146,31 +5150,31 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>VTS</t>
+          <t>APTV</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Vitesse Energy, Inc.</t>
+          <t>Aptiv PLC</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E31" s="16" t="n">
-        <v>3.874</v>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>-3</v>
+        <v>4.344</v>
+      </c>
+      <c r="F31" s="21" t="n">
+        <v>68</v>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>PSU:28 F4:5 RI:50</t>
+          <t>PSU:36 BB:5 RI:35</t>
         </is>
       </c>
     </row>
@@ -5180,22 +5184,22 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>PRGO</t>
+          <t>OPCH</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Perrigo Company plc</t>
+          <t>Option Care Health, Inc.</t>
         </is>
       </c>
       <c r="D32" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E32" s="17" t="n">
-        <v>3.846</v>
+        <v>4.26</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>-12</v>
+        <v>16</v>
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
@@ -5204,7 +5208,7 @@
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t>PSU:21 RI:48 SS:29</t>
+          <t>PSU:27 BB:5 C10:-1 F4:23 RI:52</t>
         </is>
       </c>
     </row>
@@ -5214,31 +5218,31 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>MMS</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>G-III Apparel Group, LTD.</t>
+          <t>Maximus, Inc.</t>
         </is>
       </c>
       <c r="D33" s="5" t="n">
         <v>6</v>
       </c>
       <c r="E33" s="16" t="n">
-        <v>3.822</v>
+        <v>4.182</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>-12</v>
+        <v>27</v>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>PSU:31 BB:5 RI:34</t>
+          <t>PSU:42 BB:5 RI:53 SS:26</t>
         </is>
       </c>
     </row>
@@ -5248,31 +5252,31 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>ENOV</t>
+          <t>GTM</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Enovis Corporation</t>
+          <t>ZoomInfo Technologies Inc.</t>
         </is>
       </c>
       <c r="D34" s="8" t="n">
         <v>6</v>
       </c>
       <c r="E34" s="17" t="n">
-        <v>3.766</v>
-      </c>
-      <c r="F34" s="21" t="n">
-        <v>65</v>
+        <v>4.056</v>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>27</v>
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t>PSU:22 C10:30 RI:46</t>
+          <t>PSU:36 BB:5 C10:-4 RI:66 SS:20</t>
         </is>
       </c>
     </row>
@@ -13631,7 +13635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -13661,7 +13665,7 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>Raw layers: 38    Effective-independent (rho&gt;0.6): 33</t>
+          <t>Raw layers: 39    Effective-independent (rho&gt;0.6): 34</t>
         </is>
       </c>
     </row>
@@ -14110,16 +14114,16 @@
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>valuation</t>
+          <t>post_ch11</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>financial_primary</t>
+          <t>equity_committee</t>
         </is>
       </c>
       <c r="C28" s="17" t="n">
-        <v>0.275</v>
+        <v>0.277</v>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
@@ -14130,16 +14134,16 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>f4_buys</t>
+          <t>valuation</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>bb_insider_overlay</t>
+          <t>financial_primary</t>
         </is>
       </c>
       <c r="C29" s="16" t="n">
-        <v>0.274</v>
+        <v>0.275</v>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
@@ -14150,16 +14154,16 @@
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>valuation</t>
+          <t>f4_buys</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>quarterly_10q</t>
+          <t>bb_insider_overlay</t>
         </is>
       </c>
       <c r="C30" s="17" t="n">
-        <v>0.265</v>
+        <v>0.274</v>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
@@ -14170,25 +14174,45 @@
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
+          <t>valuation</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>quarterly_10q</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
           <t>psu</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>buyback</t>
         </is>
       </c>
-      <c r="C31" s="16" t="n">
+      <c r="C32" s="17" t="n">
         <v>0.253</v>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>moderate</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>Spearman rank correlation across the full universe. Pairs above rho 0.6 are folded into a single effective layer for the independence count: PSU + Voss CIC (Voss derives from the PSU plan), the tender family (tender + mechanism + bumpitrage share one source), and Form 4 + opportunistic insiders (one refines the other). A high raw layer-firing count should be read against this: nine layers firing is closer to seven or eight genuinely independent confirmations.</t>
         </is>
@@ -14197,9 +14221,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A33:D33"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A34:D34"/>
   </mergeCells>
   <printOptions horizontalCentered="0"/>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
@@ -14346,7 +14370,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -14374,7 +14398,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -14402,7 +14426,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -14430,7 +14454,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -14458,7 +14482,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -14486,7 +14510,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -14514,7 +14538,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>7d</t>
+          <t>13d</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -14570,7 +14594,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -14598,7 +14622,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E16" s="10" t="inlineStr">
@@ -14626,7 +14650,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -14766,7 +14790,7 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>8d</t>
+          <t>14d</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -14862,7 +14886,7 @@
         <v>8</v>
       </c>
       <c r="B29" s="17" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
@@ -14875,7 +14899,7 @@
         <v>7</v>
       </c>
       <c r="B30" s="16" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
@@ -14901,7 +14925,7 @@
         <v>5</v>
       </c>
       <c r="B32" s="16" t="n">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
@@ -14914,7 +14938,7 @@
         <v>4</v>
       </c>
       <c r="B33" s="17" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
@@ -14927,7 +14951,7 @@
         <v>3</v>
       </c>
       <c r="B34" s="16" t="n">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
@@ -14940,7 +14964,7 @@
         <v>2</v>
       </c>
       <c r="B35" s="17" t="n">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
@@ -14953,7 +14977,7 @@
         <v>1</v>
       </c>
       <c r="B36" s="16" t="n">
-        <v>1241</v>
+        <v>1233</v>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
@@ -14964,7 +14988,7 @@
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>38 total scoring layers, all additive. Coverage and data age are read live from each layer's source file at build time; no figures are hardcoded. Layers with low coverage (Form 4, 13F-delta, tender) are signal-sparse by design — they fire only on names exhibiting the pattern. The layer-firing distribution is the count of names firing on N independent layers; per the correlation analysis (layer_correlation_pairs.csv) the effective-independent layer count is ~21 of 30 at rho&gt;0.6.</t>
+          <t>39 total scoring layers, all additive. Coverage and data age are read live from each layer's source file at build time; no figures are hardcoded. Layers with low coverage (Form 4, 13F-delta, tender) are signal-sparse by design — they fire only on names exhibiting the pattern. The layer-firing distribution is the count of names firing on N independent layers; per the correlation analysis (layer_correlation_pairs.csv) the effective-independent layer count is ~21 of 30 at rho&gt;0.6.</t>
         </is>
       </c>
     </row>
@@ -15186,7 +15210,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>10 layers firing | cons 8.678</t>
+          <t>10 layers firing | cons 8.874</t>
         </is>
       </c>
     </row>
@@ -15196,12 +15220,12 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>HFFG</t>
+          <t>VSNT</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>HF Foods Group</t>
+          <t>VSNT</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -15211,7 +15235,7 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Triple PSU $ hurdle (rev/EBITDA/FCF) + clawback strengthened + 4-buyer F4 cluster</t>
+          <t>9 layers firing | cons 8.776</t>
         </is>
       </c>
     </row>
@@ -15221,22 +15245,22 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>WW</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Salesforce</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>WW</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
+          <t>9 layers firing | cons 8.12</t>
         </is>
       </c>
     </row>
@@ -15246,22 +15270,22 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>DXC</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>DXC Technology</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
+          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
         </is>
       </c>
     </row>
@@ -15271,12 +15295,12 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>FOUR</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>FOUR</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -15286,7 +15310,7 @@
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 7.068</t>
+          <t>9 layers firing | cons 6.73</t>
         </is>
       </c>
     </row>
@@ -15296,22 +15320,22 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>PAR</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>POOL</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 6.958</t>
+          <t>9 layers firing | cons 6.634</t>
         </is>
       </c>
     </row>
@@ -15321,22 +15345,22 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>FOUR</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>FOUR</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>PAR</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 6.426</t>
+          <t>9 layers firing | cons 6.622</t>
         </is>
       </c>
     </row>
@@ -15371,12 +15395,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>VSNT</t>
+          <t>HFFG</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>VSNT</t>
+          <t>HF Foods Group</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -15386,7 +15410,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 7.79</t>
+          <t>Triple PSU $ hurdle (rev/EBITDA/FCF) + clawback strengthened + 4-buyer F4 cluster</t>
         </is>
       </c>
     </row>
@@ -15396,12 +15420,12 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>WW</t>
+          <t>GPK</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>WW</t>
+          <t>GPK</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -15411,7 +15435,7 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 7.152</t>
+          <t>8 layers firing | cons 7.142</t>
         </is>
       </c>
     </row>
@@ -15421,12 +15445,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>Universal Display</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -15436,7 +15460,7 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.782</t>
+          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
         </is>
       </c>
     </row>
@@ -15461,7 +15485,7 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.478</t>
+          <t>8 layers firing | cons 6.486</t>
         </is>
       </c>
     </row>
@@ -15486,7 +15510,7 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.37</t>
+          <t>8 layers firing | cons 6.428</t>
         </is>
       </c>
     </row>
@@ -15496,12 +15520,12 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Universal Display</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -15511,7 +15535,7 @@
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
+          <t>8 layers firing | cons 6.374</t>
         </is>
       </c>
     </row>
@@ -15521,22 +15545,22 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>DXC Technology</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.33</t>
+          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
         </is>
       </c>
     </row>
@@ -15546,22 +15570,22 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>PRGO</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>PRGO</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Participation 1-2%</t>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.95</t>
+          <t>8 layers firing | cons 6.152</t>
         </is>
       </c>
     </row>
@@ -15571,22 +15595,22 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>HDSN</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>GIII</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>Hudson Technologies</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.934</t>
+          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
         </is>
       </c>
     </row>
@@ -15596,22 +15620,22 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>TKO</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Zoetis</t>
-        </is>
-      </c>
-      <c r="D33" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>TKO</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>F4 cluster + valuation + recent-incentive 60% drawdown</t>
+          <t>8 layers firing | cons 5.706</t>
         </is>
       </c>
     </row>
@@ -15621,22 +15645,22 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>TKO</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>TKO</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+          <t>NSP</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.696</t>
+          <t>8 layers firing | cons 5.57</t>
         </is>
       </c>
     </row>
@@ -15646,22 +15670,22 @@
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>HDSN</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Hudson Technologies</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
+          <t>8 layers firing | cons 5.562</t>
         </is>
       </c>
     </row>
@@ -15786,7 +15810,7 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t>38 additive scoring layers ingested per ticker, spanning PSU forensics, governance, valuation, verified buybacks, tender mechanics, 10b5-1 direction, Form 4 (raw + Cohen-Malloy opportunistic), Form 144, quarterly 10-Q, NCAV, Voss CIC, post-Ch11, internalization, bumpitrage, spinoff timing, Arquitos, Coval-Stafford proxy + real N-PORT, backstopped rights, FDIC dark banks, activist letters, 13F-delta, biotech PDUFA, financial-sector primary, discretionary insider conviction, emergence cross-feed, Sohn pitches, asymmetry assembly (PSIX recipe), distressed-stub progress, premium injections, selective buybacks, and hidden-asset realisation.</t>
+          <t>39 additive scoring layers ingested per ticker, spanning PSU forensics, governance, valuation, verified buybacks, tender mechanics, 10b5-1 direction, Form 4 (raw + Cohen-Malloy opportunistic), Form 144, quarterly 10-Q, NCAV, Voss CIC, post-Ch11, internalization, bumpitrage, spinoff timing, Arquitos, Coval-Stafford proxy + real N-PORT, backstopped rights, FDIC dark banks, activist letters, 13F-delta, biotech PDUFA, financial-sector primary, discretionary insider conviction, emergence cross-feed, Sohn pitches, asymmetry assembly (PSIX recipe), distressed-stub progress, premium injections, selective buybacks, and hidden-asset realisation.</t>
         </is>
       </c>
     </row>
@@ -15876,7 +15900,7 @@
       </c>
       <c r="C12" s="26" t="inlineStr">
         <is>
-          <t>Pairwise Spearman correlation (layer_correlation_pairs.csv) collapses 38 raw layers to effective-independent at rho&gt;0.6. Three correlated clusters: PSU+Voss, tender family, F4+opportunistic. 'Fires 9 layers' ≈ 7-8 true confirmations.</t>
+          <t>Pairwise Spearman correlation (layer_correlation_pairs.csv) collapses 39 raw layers to effective-independent at rho&gt;0.6. Three correlated clusters: PSU+Voss, tender family, F4+opportunistic. 'Fires 9 layers' ≈ 7-8 true confirmations.</t>
         </is>
       </c>
     </row>
@@ -16086,7 +16110,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>10 layers firing | cons 8.678</t>
+          <t>10 layers firing | cons 8.874</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -16103,39 +16127,39 @@
     <row r="6" ht="56" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>HFFG</t>
+          <t>VSNT</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>HF Foods Group</t>
+          <t>VSNT</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>101</v>
+        <v>5407</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>1.89</v>
+        <v>38.21</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>0.49</v>
+        <v>0.54</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>revenue_dollar_target</t>
+          <t>spin_separation</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>Triple PSU $ hurdle (rev/EBITDA/FCF) + clawback strengthened + 4-buyer F4 cluster</t>
+          <t>9 layers firing | cons 8.776</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>P/B 0.48 + microcap distributor with hard assets</t>
+          <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
@@ -16147,69 +16171,69 @@
     <row r="7" ht="56" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>WW</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Salesforce</t>
+          <t>WW</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>124308</v>
+        <v>192</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>151.78</v>
+        <v>19.2</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>3.63</v>
+        <v>0.6</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>chapter11_emergence</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
+          <t>9 layers firing | cons 8.12</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Mega-cap recurring revenue base</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>see proxy_scan + buyback_verify</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="8" ht="56" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>DXC</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>DXC Technology</t>
+          <t>Salesforce</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1394</v>
+        <v>124308</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>8.6</v>
+        <v>151.78</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>0.48</v>
+        <v>3.63</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
@@ -16218,51 +16242,51 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
+          <t>PSU + buyback + recent 10b5-1 termination + F4 cluster</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>IT services franchise; transformation signal in PSU</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>Participation 1-2%</t>
+          <t>Mega-cap recurring revenue base</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
     <row r="9" ht="56" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>FOUR</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>FOUR</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>7252</v>
+        <v>3906</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>198.99</v>
+        <v>39.4</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>6.4</v>
+        <v>4.82</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>fda_phase_milestone</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 7.068</t>
+          <t>9 layers firing | cons 6.73</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
@@ -16279,34 +16303,34 @@
     <row r="10" ht="56" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>PAR</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>631</v>
+        <v>7252</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>15.29</v>
+        <v>198.99</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>0.76</v>
+        <v>6.4</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>fda_phase_milestone</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 6.958</t>
+          <t>9 layers firing | cons 6.634</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
@@ -16314,34 +16338,34 @@
           <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="11" ht="56" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>FOUR</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>FOUR</t>
+          <t>PAR</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>3906</v>
+        <v>631</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>39.4</v>
+        <v>15.29</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>4.82</v>
+        <v>0.76</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
@@ -16350,7 +16374,7 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>9 layers firing | cons 6.426</t>
+          <t>9 layers firing | cons 6.622</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -16358,9 +16382,9 @@
           <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
@@ -16411,39 +16435,39 @@
     <row r="13" ht="56" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>VSNT</t>
+          <t>HFFG</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>VSNT</t>
+          <t>HF Foods Group</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>5407</v>
+        <v>101</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>38.21</v>
+        <v>1.89</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>0.54</v>
+        <v>0.49</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>spin_separation</t>
+          <t>revenue_dollar_target</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 7.79</t>
+          <t>Triple PSU $ hurdle (rev/EBITDA/FCF) + clawback strengthened + 4-buyer F4 cluster</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
+          <t>P/B 0.48 + microcap distributor with hard assets</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -16455,34 +16479,34 @@
     <row r="14" ht="56" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>WW</t>
+          <t>GPK</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>WW</t>
+          <t>GPK</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>192</v>
+        <v>3169</v>
       </c>
       <c r="D14" s="17" t="n">
-        <v>19.2</v>
+        <v>10.71</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>0.6</v>
+        <v>0.98</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>chapter11_emergence</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 7.152</t>
+          <t>8 layers firing | cons 7.142</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -16499,39 +16523,39 @@
     <row r="15" ht="56" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>OLED</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>HUBS</t>
+          <t>Universal Display</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
-        <v>9011</v>
+        <v>4158</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>176.03</v>
+        <v>88.94</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>4.58</v>
+        <v>2.44</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>revenue_dollar_target</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.782</t>
+          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
+          <t>OLED IP moat</t>
         </is>
       </c>
       <c r="J15" s="6" t="inlineStr">
@@ -16570,7 +16594,7 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.478</t>
+          <t>8 layers firing | cons 6.486</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
@@ -16614,7 +16638,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.37</t>
+          <t>8 layers firing | cons 6.428</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
@@ -16631,39 +16655,39 @@
     <row r="18" ht="56" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Universal Display</t>
+          <t>GPGI</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>4158</v>
+        <v>4180</v>
       </c>
       <c r="D18" s="17" t="n">
-        <v>88.94</v>
+        <v>14.42</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>2.44</v>
+        <v>1.34</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>revenue_dollar_target</t>
+          <t>spin_separation</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>PSU + F4 cluster + recent-incentive 60% drawdown</t>
+          <t>8 layers firing | cons 6.374</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>OLED IP moat</t>
+          <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
@@ -16675,69 +16699,69 @@
     <row r="19" ht="56" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>DXC Technology</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>4180</v>
+        <v>1394</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>14.42</v>
+        <v>8.6</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>1.34</v>
+        <v>0.48</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>spin_separation</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 6.33</t>
+          <t>PSU core 40 + buyback + recent-incentive 57% drawdown</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
+          <t>IT services franchise; transformation signal in PSU</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
     <row r="20" ht="56" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>PRGO</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>PRGO</t>
+          <t>HUBS</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>1418</v>
+        <v>9011</v>
       </c>
       <c r="D20" s="17" t="n">
-        <v>10.25</v>
+        <v>176.03</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>0.57</v>
+        <v>4.58</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
@@ -16746,7 +16770,7 @@
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.95</t>
+          <t>8 layers firing | cons 6.152</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
@@ -16756,32 +16780,34 @@
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>Participation 1-2%</t>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="21" ht="56" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>HDSN</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>Hudson Technologies</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
-        <v>1467</v>
+        <v>222</v>
       </c>
       <c r="D21" s="16" t="n">
-        <v>34.77</v>
+        <v>5.27</v>
       </c>
       <c r="E21" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>33</v>
+        <v>0.93</v>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
@@ -16790,42 +16816,42 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.934</t>
+          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>see proxy_scan + buyback_verify</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>Refrigerant reclaim regulatory moat</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="22" ht="56" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>ZTS</t>
+          <t>TKO</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Zoetis</t>
+          <t>TKO</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>32997</v>
+        <v>37992</v>
       </c>
       <c r="D22" s="17" t="n">
-        <v>78.70999999999999</v>
+        <v>198.78</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>10.04</v>
+        <v>4.41</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
@@ -16834,51 +16860,51 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>F4 cluster + valuation + recent-incentive 60% drawdown</t>
+          <t>8 layers firing | cons 5.706</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>Animal health franchise</t>
-        </is>
-      </c>
-      <c r="J22" s="10" t="inlineStr">
-        <is>
-          <t>Material 2-5%</t>
+          <t>see proxy_scan + buyback_verify</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>Concentrated 5%+</t>
         </is>
       </c>
     </row>
     <row r="23" ht="56" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>TKO</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>TKO</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
-        <v>37992</v>
+        <v>1382</v>
       </c>
       <c r="D23" s="16" t="n">
-        <v>198.78</v>
+        <v>36.22</v>
       </c>
       <c r="E23" s="16" t="n">
-        <v>4.41</v>
+        <v>20.64</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>ebitda_dollar_target</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>8 layers firing | cons 5.696</t>
+          <t>8 layers firing | cons 5.57</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
@@ -16886,31 +16912,31 @@
           <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>Concentrated 5%+</t>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>Material 2-5%</t>
         </is>
       </c>
     </row>
     <row r="24" ht="56" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>HDSN</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Hudson Technologies</t>
+          <t>LULU</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>222</v>
+        <v>13781</v>
       </c>
       <c r="D24" s="17" t="n">
-        <v>5.27</v>
+        <v>121.36</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>0.93</v>
+        <v>2.85</v>
       </c>
       <c r="F24" s="10" t="inlineStr">
         <is>
@@ -16924,17 +16950,17 @@
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>Recent F4 cluster + buyback + special-sits + recent-incentive</t>
+          <t>8 layers firing | cons 5.562</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr">
         <is>
-          <t>Refrigerant reclaim regulatory moat</t>
+          <t>see proxy_scan + buyback_verify</t>
         </is>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>Concentrated 5%+</t>
+          <t>Participation 1-2%</t>
         </is>
       </c>
     </row>
@@ -19269,7 +19295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -19561,7 +19587,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>OSUR</t>
         </is>
       </c>
       <c r="C15" s="16" t="n">
@@ -19569,12 +19595,12 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>front-loaded grant</t>
+          <t>discretionary hurdle, repricing language, single-trigger CIC</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Concentrate (1 flag tolerable)</t>
+          <t>Participation — limited size</t>
         </is>
       </c>
     </row>
@@ -19584,7 +19610,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>OSUR</t>
+          <t>SD</t>
         </is>
       </c>
       <c r="C16" s="17" t="n">
@@ -19592,12 +19618,12 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>discretionary hurdle, repricing language, single-trigger CIC</t>
+          <t>front-loaded grant</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Participation — limited size</t>
+          <t>Concentrate (1 flag tolerable)</t>
         </is>
       </c>
     </row>
@@ -19630,7 +19656,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>GWW</t>
         </is>
       </c>
       <c r="C18" s="17" t="n">
@@ -19653,7 +19679,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>GWW</t>
+          <t>ADT</t>
         </is>
       </c>
       <c r="C19" s="16" t="n">
@@ -19676,7 +19702,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>ADT</t>
+          <t>SAFE</t>
         </is>
       </c>
       <c r="C20" s="17" t="n">
@@ -19684,7 +19710,7 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>retirement carveout</t>
+          <t>front-loaded grant</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -19699,7 +19725,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>SAFE</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="C21" s="16" t="n">
@@ -19707,12 +19733,12 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>front-loaded grant</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>Concentrate (1 flag tolerable)</t>
+          <t>front-loaded grant, retirement carveout</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Material — basket diversify</t>
         </is>
       </c>
     </row>
@@ -19722,15 +19748,15 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FISV</t>
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>front-loaded grant, retirement carveout</t>
+          <t>repricing language, retirement carveout</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -19745,7 +19771,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>FISV</t>
+          <t>TROX</t>
         </is>
       </c>
       <c r="C23" s="16" t="n">
@@ -19753,12 +19779,12 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>repricing language, retirement carveout</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Material — basket diversify</t>
+          <t>retirement carveout</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Concentrate (1 flag tolerable)</t>
         </is>
       </c>
     </row>
@@ -19768,7 +19794,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>TROX</t>
+          <t>CNMD</t>
         </is>
       </c>
       <c r="C24" s="17" t="n">
@@ -19776,7 +19802,7 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>retirement carveout</t>
+          <t>repricing language</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -19791,7 +19817,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>CNMD</t>
+          <t>BEEP</t>
         </is>
       </c>
       <c r="C25" s="16" t="n">
@@ -19799,7 +19825,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>repricing language</t>
+          <t>retirement carveout</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -19814,7 +19840,7 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>BEEP</t>
+          <t>DXLG</t>
         </is>
       </c>
       <c r="C26" s="17" t="n">
@@ -19837,7 +19863,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>DXLG</t>
+          <t>KMPR</t>
         </is>
       </c>
       <c r="C27" s="16" t="n">
@@ -19845,12 +19871,12 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>retirement carveout</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Concentrate (1 flag tolerable)</t>
+          <t>repricing language, retirement carveout</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Material — basket diversify</t>
         </is>
       </c>
     </row>
@@ -19860,7 +19886,7 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>KMPR</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="C28" s="17" t="n">
@@ -19883,7 +19909,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>DXC</t>
         </is>
       </c>
       <c r="C29" s="16" t="n">
@@ -19891,12 +19917,12 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>repricing language, retirement carveout</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>Material — basket diversify</t>
+          <t>discretionary hurdle, repricing language, retirement carveout</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Participation — limited size</t>
         </is>
       </c>
     </row>
@@ -19906,7 +19932,7 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>DXC</t>
+          <t>PSN</t>
         </is>
       </c>
       <c r="C30" s="17" t="n">
@@ -19914,12 +19940,12 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>discretionary hurdle, repricing language, retirement carveout</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Participation — limited size</t>
+          <t>repricing language, retirement carveout</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>Material — basket diversify</t>
         </is>
       </c>
     </row>
@@ -19929,7 +19955,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>PSN</t>
+          <t>LGL</t>
         </is>
       </c>
       <c r="C31" s="16" t="n">
@@ -19937,12 +19963,12 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>repricing language, retirement carveout</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>Material — basket diversify</t>
+          <t>repricing language</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Concentrate (1 flag tolerable)</t>
         </is>
       </c>
     </row>
@@ -19952,7 +19978,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>LGL</t>
+          <t>WHR</t>
         </is>
       </c>
       <c r="C32" s="17" t="n">
@@ -19960,12 +19986,12 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>repricing language</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Concentrate (1 flag tolerable)</t>
+          <t>repricing language, retirement carveout</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>Material — basket diversify</t>
         </is>
       </c>
     </row>
@@ -19975,7 +20001,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>WHR</t>
+          <t>TBI</t>
         </is>
       </c>
       <c r="C33" s="16" t="n">
@@ -19983,7 +20009,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>repricing language, retirement carveout</t>
+          <t>discretionary hurdle, retirement carveout</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -19998,7 +20024,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>WW</t>
+          <t>POOL</t>
         </is>
       </c>
       <c r="C34" s="17" t="n">
@@ -20021,7 +20047,7 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>TBI</t>
+          <t>WW</t>
         </is>
       </c>
       <c r="C35" s="16" t="n">
@@ -20029,12 +20055,12 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>discretionary hurdle, retirement carveout</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>Material — basket diversify</t>
+          <t>retirement carveout</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Concentrate (1 flag tolerable)</t>
         </is>
       </c>
     </row>
@@ -20044,7 +20070,7 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>OPCH</t>
         </is>
       </c>
       <c r="C36" s="17" t="n">
@@ -20521,8 +20547,31 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="28" customHeight="1">
-      <c r="A58" s="11" t="inlineStr">
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="5" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>NXT</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>repricing language, retirement carveout</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Material — basket diversify</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="28" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>Eight flag classes: single-trigger CIC, repricing language, retirement carveout, front-loaded grant, discretionary hurdle, aggregate-only metrics, plus structural variants. Counter-intuitive: a 'repricing language' flag can become a re-rate catalyst when a stock has fallen sharply, since management becomes incentivised to reset hurdles. Read the flag in context, not as automatic veto.</t>
         </is>
@@ -20531,8 +20580,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A58:E58"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A59:E59"/>
   </mergeCells>
   <printOptions horizontalCentered="0"/>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
@@ -24178,7 +24227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -24419,12 +24468,12 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>HFFG</t>
+          <t>GPK</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>HF Foods Group Inc.</t>
+          <t>Graphic Packaging Holdin</t>
         </is>
       </c>
       <c r="C7" s="16" t="n">
@@ -24482,19 +24531,19 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>SMRT</t>
+          <t>HFFG</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>SmartRent, Inc.</t>
+          <t>HF Foods Group Inc.</t>
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
@@ -24503,7 +24552,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>●</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -24523,14 +24572,14 @@
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
           <t>●</t>
         </is>
       </c>
-      <c r="K8" s="10" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
       <c r="L8" s="10" t="inlineStr">
         <is>
           <t>–</t>
@@ -24538,84 +24587,588 @@
       </c>
       <c r="M8" s="10" t="inlineStr">
         <is>
-          <t>4/8 components</t>
+          <t>5/8 components converge</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>GLP</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Global Partners LP</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>4/8 components</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>SMRT</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>SmartRent, Inc.</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>44</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M10" s="10" t="inlineStr">
+        <is>
+          <t>4/8 components</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>GPN</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Global Payments Inc.</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>41</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>4/8 components</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>BCIC</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>BCP Investment Corporati</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>37</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>4/8 components</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>PTLO</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Portillo's Inc.</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>4/8 components</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>NSP</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Insperity, Inc.</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="n">
+        <v>37</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F14" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L14" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M14" s="10" t="inlineStr">
+        <is>
+          <t>4/8 components</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t>PAL</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Proficient Auto Logistic</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C15" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D15" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>●</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="L9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>5 names pass the assembly SPINE (top 45 shown): low expectations AND an engine (operating inflection or leverage torque) AND a costly-action alignment signal (open-market insider buy or a curated maturity-extension / subordination event). A name strong on many unrelated layers but missing a spine leg scores ZERO here — that is the point: asymmetry is a conjunction, not a sum. Components: Cheap (C1, incl. EV/EBIT), Lev (C2 survivable leverage), Orph (C3 drawdown/orphaned), Insdr (C4 open-market buys), Catl (C5 emergence/tender/activist), Inflx (C6 gross profit up while revenue down / margin expansion, from XBRL), Delev (C7 debt &amp; interest falling), Cap (C8 low capex + high marginal returns). Convergence beyond the spine adds a convexity bonus; dilutive-refinancing / backstop-expiry counter-signals subtract. The engine is validated point-in-time: it flags May-2024 PSIX (@ $2.15, 7/8 components) — see asymmetry_backtest.py. Source: asymmetry_assembly.json (+ financials_inflection.json XBRL).</t>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>VSNT</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Versant Media Group, Inc</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L16" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M16" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>LCNB</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>LCNB Corporation</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>●</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>13 names pass the assembly SPINE (top 45 shown): low expectations AND an engine (operating inflection or leverage torque) AND a costly-action alignment signal (open-market insider buy or a curated maturity-extension / subordination event). A name strong on many unrelated layers but missing a spine leg scores ZERO here — that is the point: asymmetry is a conjunction, not a sum. Components: Cheap (C1, incl. EV/EBIT), Lev (C2 survivable leverage), Orph (C3 drawdown/orphaned), Insdr (C4 open-market buys), Catl (C5 emergence/tender/activist), Inflx (C6 gross profit up while revenue down / margin expansion, from XBRL), Delev (C7 debt &amp; interest falling), Cap (C8 low capex + high marginal returns). Convergence beyond the spine adds a convexity bonus; dilutive-refinancing / backstop-expiry counter-signals subtract. The engine is validated point-in-time: it flags May-2024 PSIX (@ $2.15, 7/8 components) — see asymmetry_backtest.py. Source: asymmetry_assembly.json (+ financials_inflection.json XBRL).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A19:M19"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A11:M11"/>
     <mergeCell ref="A1:M1"/>
   </mergeCells>
   <printOptions horizontalCentered="0"/>

</xml_diff>

<commit_message>
Regenerate MOST_ASYMMETRIC.xlsx; surface the Form 4 filing-time layer
The workbook builder's Methodology prose predated several layers. Update
it to name the net-buyback, Lynch-reawakening, and Form 4 filing-TIME
signals in the layer-ingestion list, replace the hardcoded "30 layers"
with the live count (now 42), and revise the honest-limitations note:
the filing-time layer is the one return-validated exception (+3.7% vs
-8.0% median, off-hours vs market-hours). Book regenerated (20 tabs).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017dpaFdbqUZj62BWE6zHYXu
</commit_message>
<xml_diff>
--- a/MOST_ASYMMETRIC.xlsx
+++ b/MOST_ASYMMETRIC.xlsx
@@ -15838,7 +15838,7 @@
       </c>
       <c r="C6" s="26" t="inlineStr">
         <is>
-          <t>42 additive scoring layers ingested per ticker, spanning PSU forensics, governance, valuation, verified buybacks, tender mechanics, 10b5-1 direction, Form 4 (raw + Cohen-Malloy opportunistic), Form 144, quarterly 10-Q, NCAV, Voss CIC, post-Ch11, internalization, bumpitrage, spinoff timing, Arquitos, Coval-Stafford proxy + real N-PORT, backstopped rights, FDIC dark banks, activist letters, 13F-delta, biotech PDUFA, financial-sector primary, discretionary insider conviction, emergence cross-feed, Sohn pitches, asymmetry assembly (PSIX recipe), distressed-stub progress, premium injections, selective buybacks, and hidden-asset realisation.</t>
+          <t>42 additive scoring layers ingested per ticker, spanning PSU forensics, governance, valuation, verified buybacks, tender mechanics, 10b5-1 direction, Form 4 (raw + Cohen-Malloy opportunistic), Form 144, quarterly 10-Q, NCAV, Voss CIC, post-Ch11, internalization, bumpitrage, spinoff timing, Arquitos, Coval-Stafford proxy + real N-PORT, backstopped rights, FDIC dark banks, activist letters, 13F-delta, biotech PDUFA, financial-sector primary, discretionary insider conviction, emergence cross-feed, Sohn pitches, asymmetry assembly (PSIX recipe), distressed-stub progress, premium injections, selective buybacks, hidden-asset realisation, net buyback (diluted-share reduction net of SBC), the Lynch reawakening momentum leg, and the Form 4 filing-TIME signal (off-hours / Friday-evening open-market buys = quiet accumulators followed; market-hours buys = price support, faded).</t>
         </is>
       </c>
     </row>
@@ -15913,7 +15913,7 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>n_layers_firing = how many of the 30 independent layers produce a non-zero score for the ticker. consensus_score = sum of per-layer rank-decay contributions across the universe.</t>
+          <t>n_layers_firing = how many of the 42 independent layers produce a non-zero score for the ticker. consensus_score = sum of per-layer rank-decay contributions across the universe.</t>
         </is>
       </c>
     </row>
@@ -15988,7 +15988,7 @@
       </c>
       <c r="C16" s="26" t="inlineStr">
         <is>
-          <t>No realized-return backtest yet (AUDIT.md S1.1) — the composite is a structurally-sound pattern-recognition system, not yet validated alpha. Cohen-Malloy needs deeper Form 4 history. Coval-Stafford proxy supplements but does not replace the N-PORT real signal. See AUDIT.md for the full ledger.</t>
+          <t>Most layers are not yet return-validated (AUDIT.md S1.1) — the composite is a structurally-sound pattern-recognition system, not yet validated alpha. The one exception is the Form 4 filing-time layer, built FROM a measured test: off-hours buys showed a +3.7% median vs -8.0% for market-hours buys (+11.7pp differential, buy-to-now proxy). Cohen-Malloy needs deeper Form 4 history. Coval-Stafford proxy supplements but does not replace the N-PORT real signal. See AUDIT.md for the full ledger.</t>
         </is>
       </c>
     </row>

</xml_diff>